<commit_message>
Added compressor and CPu
</commit_message>
<xml_diff>
--- a/adopt_net0/database/templates/technology_data/Industrial/CementHybridCCS_data/cement_sheet.xlsx
+++ b/adopt_net0/database/templates/technology_data/Industrial/CementHybridCCS_data/cement_sheet.xlsx
@@ -8,15 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\AdOpT-NET0\adopt_net0\database\templates\technology_data\Industrial\CementHybridCCS_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAC3FA7B-B280-4278-B89C-46542FB039ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{791A84AB-DAFF-4197-9592-1CBD599E4F2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-180" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{C0ECAA26-0769-408D-9398-31AECF4E3649}"/>
+    <workbookView xWindow="-28920" yWindow="-180" windowWidth="29040" windowHeight="15840" activeTab="5" xr2:uid="{C0ECAA26-0769-408D-9398-31AECF4E3649}"/>
   </bookViews>
   <sheets>
-    <sheet name="oxyfuel" sheetId="1" r:id="rId1"/>
-    <sheet name="mea" sheetId="2" r:id="rId2"/>
-    <sheet name="other_data" sheetId="3" r:id="rId3"/>
-    <sheet name="calculations" sheetId="4" r:id="rId4"/>
+    <sheet name="capex_oxyfuel" sheetId="1" r:id="rId1"/>
+    <sheet name="capex_mea" sheetId="2" r:id="rId2"/>
+    <sheet name="capex_cpu_oxyfuel" sheetId="6" r:id="rId3"/>
+    <sheet name="capex_compressor_mea" sheetId="5" r:id="rId4"/>
+    <sheet name="energy_oxy_mea" sheetId="3" r:id="rId5"/>
+    <sheet name="energy_cpu_compressor" sheetId="7" r:id="rId6"/>
+    <sheet name="calculations" sheetId="4" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="68">
   <si>
     <t>size_tclinker_per_h</t>
   </si>
@@ -295,6 +298,24 @@
   <si>
     <t>value</t>
   </si>
+  <si>
+    <t>el_cons_cpu</t>
+  </si>
+  <si>
+    <t>electricity_cons_MWh/tCO2</t>
+  </si>
+  <si>
+    <t>liquid</t>
+  </si>
+  <si>
+    <t>gas</t>
+  </si>
+  <si>
+    <t>supercritical</t>
+  </si>
+  <si>
+    <t>el_cons_compressor</t>
+  </si>
 </sst>
 </file>
 
@@ -303,7 +324,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -353,6 +374,12 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -540,7 +567,7 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -598,6 +625,11 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="3" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Calculation" xfId="5" builtinId="22"/>
@@ -978,6 +1010,7 @@
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -991,7 +1024,8 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>3.75</v>
+        <f>calculations!D15</f>
+        <v>3.7084942228242932</v>
       </c>
       <c r="B2">
         <f>calculations!D16</f>
@@ -1000,7 +1034,8 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>12.51</v>
+        <f>calculations!G15</f>
+        <v>12.361647409414312</v>
       </c>
       <c r="B3">
         <f>calculations!G16</f>
@@ -1009,7 +1044,8 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>20.85</v>
+        <f>calculations!G6</f>
+        <v>20.602745682357188</v>
       </c>
       <c r="B4">
         <f>calculations!G7</f>
@@ -1023,6 +1059,141 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E17DFFB0-96B6-4F96-B3DF-E2D36B37C43F}">
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>75</v>
+      </c>
+      <c r="B2">
+        <v>48600000</v>
+      </c>
+      <c r="C2">
+        <v>50200000</v>
+      </c>
+      <c r="D2">
+        <v>61000000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>125</v>
+      </c>
+      <c r="B3">
+        <v>62500000</v>
+      </c>
+      <c r="C3">
+        <v>63300000</v>
+      </c>
+      <c r="D3">
+        <v>71600000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8995DE27-F5E7-40F1-8502-5CC793EB5921}">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <f>calculations!D15</f>
+        <v>3.7084942228242932</v>
+      </c>
+      <c r="B2">
+        <v>7530000</v>
+      </c>
+      <c r="C2">
+        <f>8.00649089380739*10^6</f>
+        <v>8006490.8938073898</v>
+      </c>
+      <c r="D2">
+        <f>10.684945673991*10^6</f>
+        <v>10684945.673991</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <f>calculations!G15</f>
+        <v>12.361647409414312</v>
+      </c>
+      <c r="B3">
+        <f>11.2041255209316*10^6</f>
+        <v>11204125.5209316</v>
+      </c>
+      <c r="C3">
+        <f>12.5665678479893*10^6</f>
+        <v>12566567.847989298</v>
+      </c>
+      <c r="D3">
+        <f>16.5887397694844*10^6</f>
+        <v>16588739.769484399</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <f>calculations!G6</f>
+        <v>20.602745682357188</v>
+      </c>
+      <c r="B4">
+        <f>13.2435084663724*10^6</f>
+        <v>13243508.466372401</v>
+      </c>
+      <c r="C4">
+        <f>15.1282369696705*10^6</f>
+        <v>15128236.969670501</v>
+      </c>
+      <c r="D4">
+        <f>19.9398066221897*10^6</f>
+        <v>19939806.622189701</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69712579-C7D8-42EE-9801-1FD637D0A17F}">
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1064,7 +1235,71 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21185F42-04E5-4941-B133-36036095D1EF}">
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="25" t="s">
+        <v>62</v>
+      </c>
+      <c r="B2" s="26">
+        <v>0.17050594000000002</v>
+      </c>
+      <c r="C2" s="26">
+        <v>0.120245032</v>
+      </c>
+      <c r="D2" s="26">
+        <v>0.13739152500000001</v>
+      </c>
+      <c r="E2" s="25"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="25" t="s">
+        <v>67</v>
+      </c>
+      <c r="B3" s="27">
+        <v>0.11930297990344463</v>
+      </c>
+      <c r="C3" s="27">
+        <v>7.4589551950173874E-2</v>
+      </c>
+      <c r="D3" s="27">
+        <v>8.9737128657946114E-2</v>
+      </c>
+      <c r="E3" s="25"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="25"/>
+      <c r="B4" s="25"/>
+      <c r="C4" s="25"/>
+      <c r="D4" s="25"/>
+      <c r="E4" s="25"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB78D47C-565F-4352-814A-A37F11C35FBF}">
   <dimension ref="A1:T55"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2705,6 +2940,14 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A10:G10"/>
+    <mergeCell ref="A11:B14"/>
+    <mergeCell ref="C11:G11"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="G13:G14"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:B5"/>
     <mergeCell ref="C2:G2"/>
@@ -2713,14 +2956,6 @@
     <mergeCell ref="E4:E5"/>
     <mergeCell ref="F4:F5"/>
     <mergeCell ref="G4:G5"/>
-    <mergeCell ref="A10:G10"/>
-    <mergeCell ref="A11:B14"/>
-    <mergeCell ref="C11:G11"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="F13:F14"/>
-    <mergeCell ref="G13:G14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added CAPEX and OPEX of compressor and CPU
</commit_message>
<xml_diff>
--- a/adopt_net0/database/templates/technology_data/Industrial/CementHybridCCS_data/cement_sheet.xlsx
+++ b/adopt_net0/database/templates/technology_data/Industrial/CementHybridCCS_data/cement_sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\AdOpT-NET0\adopt_net0\database\templates\technology_data\Industrial\CementHybridCCS_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{791A84AB-DAFF-4197-9592-1CBD599E4F2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C1A2A18-7943-4B3D-9E3F-F96EF1E288A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-180" windowWidth="29040" windowHeight="15840" activeTab="5" xr2:uid="{C0ECAA26-0769-408D-9398-31AECF4E3649}"/>
+    <workbookView xWindow="22932" yWindow="-4404" windowWidth="30936" windowHeight="16896" activeTab="2" xr2:uid="{C0ECAA26-0769-408D-9398-31AECF4E3649}"/>
   </bookViews>
   <sheets>
     <sheet name="capex_oxyfuel" sheetId="1" r:id="rId1"/>
@@ -589,6 +589,11 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="3" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -625,11 +630,6 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="3" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Calculation" xfId="5" builtinId="22"/>
@@ -970,13 +970,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D08EB36-8885-41F7-B3E9-60083815A79B}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -984,7 +984,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>75</v>
       </c>
@@ -992,7 +992,7 @@
         <v>137540000</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>125</v>
       </c>
@@ -1008,13 +1008,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{447E0F8A-1C59-405C-B3D0-EB533A2330E6}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -1022,7 +1022,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2">
         <f>calculations!D15</f>
         <v>3.7084942228242932</v>
@@ -1032,7 +1032,7 @@
         <v>28210000.000000007</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3">
         <f>calculations!G15</f>
         <v>12.361647409414312</v>
@@ -1042,7 +1042,7 @@
         <v>46360000.000000015</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4">
         <f>calculations!G6</f>
         <v>20.602745682357188</v>
@@ -1060,10 +1060,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E17DFFB0-96B6-4F96-B3DF-E2D36B37C43F}">
-  <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -1077,31 +1077,45 @@
         <v>66</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3">
         <v>75</v>
       </c>
-      <c r="B2">
+      <c r="B3">
         <v>48600000</v>
       </c>
-      <c r="C2">
+      <c r="C3">
         <v>50200000</v>
       </c>
-      <c r="D2">
+      <c r="D3">
         <v>61000000</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4">
         <v>125</v>
       </c>
-      <c r="B3">
+      <c r="B4">
         <v>62500000</v>
       </c>
-      <c r="C3">
+      <c r="C4">
         <v>63300000</v>
       </c>
-      <c r="D3">
+      <c r="D4">
         <v>71600000</v>
       </c>
     </row>
@@ -1112,16 +1126,16 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8995DE27-F5E7-40F1-8502-5CC793EB5921}">
-  <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -1135,55 +1149,69 @@
         <v>66</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3">
         <f>calculations!D15</f>
         <v>3.7084942228242932</v>
       </c>
-      <c r="B2">
+      <c r="B3">
         <v>7530000</v>
       </c>
-      <c r="C2">
+      <c r="C3">
         <f>8.00649089380739*10^6</f>
         <v>8006490.8938073898</v>
       </c>
-      <c r="D2">
+      <c r="D3">
         <f>10.684945673991*10^6</f>
         <v>10684945.673991</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4">
         <f>calculations!G15</f>
         <v>12.361647409414312</v>
       </c>
-      <c r="B3">
+      <c r="B4">
         <f>11.2041255209316*10^6</f>
         <v>11204125.5209316</v>
       </c>
-      <c r="C3">
+      <c r="C4">
         <f>12.5665678479893*10^6</f>
         <v>12566567.847989298</v>
       </c>
-      <c r="D3">
+      <c r="D4">
         <f>16.5887397694844*10^6</f>
         <v>16588739.769484399</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5">
         <f>calculations!G6</f>
         <v>20.602745682357188</v>
       </c>
-      <c r="B4">
+      <c r="B5">
         <f>13.2435084663724*10^6</f>
         <v>13243508.466372401</v>
       </c>
-      <c r="C4">
+      <c r="C5">
         <f>15.1282369696705*10^6</f>
         <v>15128236.969670501</v>
       </c>
-      <c r="D4">
+      <c r="D5">
         <f>19.9398066221897*10^6</f>
         <v>19939806.622189701</v>
       </c>
@@ -1196,14 +1224,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69712579-C7D8-42EE-9801-1FD637D0A17F}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>58</v>
       </c>
@@ -1212,7 +1240,7 @@
         <v>0.25548249251013122</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>59</v>
       </c>
@@ -1221,7 +1249,7 @@
         <v>8.2307186539958971E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>60</v>
       </c>
@@ -1238,12 +1266,12 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21185F42-04E5-4941-B133-36036095D1EF}">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>63</v>
       </c>
@@ -1257,42 +1285,42 @@
         <v>66</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="B2" s="26">
+      <c r="B2" s="14">
         <v>0.17050594000000002</v>
       </c>
-      <c r="C2" s="26">
+      <c r="C2" s="14">
         <v>0.120245032</v>
       </c>
-      <c r="D2" s="26">
+      <c r="D2" s="14">
         <v>0.13739152500000001</v>
       </c>
-      <c r="E2" s="25"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="25" t="s">
+      <c r="E2" s="13"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="B3" s="27">
+      <c r="B3" s="15">
         <v>0.11930297990344463</v>
       </c>
-      <c r="C3" s="27">
+      <c r="C3" s="15">
         <v>7.4589551950173874E-2</v>
       </c>
-      <c r="D3" s="27">
+      <c r="D3" s="15">
         <v>8.9737128657946114E-2</v>
       </c>
-      <c r="E3" s="25"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="25"/>
-      <c r="B4" s="25"/>
-      <c r="C4" s="25"/>
-      <c r="D4" s="25"/>
-      <c r="E4" s="25"/>
+      <c r="E3" s="13"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="13"/>
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1302,23 +1330,23 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB78D47C-565F-4352-814A-A37F11C35FBF}">
   <dimension ref="A1:T55"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="52" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:20" ht="16.2" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="15"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="18"/>
       <c r="N1" s="11"/>
       <c r="O1" s="11" t="s">
         <v>50</v>
@@ -1329,18 +1357,18 @@
       <c r="S1" s="11"/>
       <c r="T1" s="3"/>
     </row>
-    <row r="2" spans="1:20" ht="18" x14ac:dyDescent="0.35">
-      <c r="A2" s="16" t="s">
+    <row r="2" spans="1:20" ht="15.6" x14ac:dyDescent="0.35">
+      <c r="A2" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="22" t="s">
+      <c r="B2" s="20"/>
+      <c r="C2" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="23"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="26"/>
       <c r="N2" s="3"/>
       <c r="O2" s="3" t="s">
         <v>27</v>
@@ -1361,9 +1389,9 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A3" s="18"/>
-      <c r="B3" s="19"/>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A3" s="21"/>
+      <c r="B3" s="22"/>
       <c r="C3" s="1" t="s">
         <v>6</v>
       </c>
@@ -1401,22 +1429,22 @@
         <v>3000.20095584</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A4" s="18"/>
-      <c r="B4" s="19"/>
-      <c r="C4" s="24">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A4" s="21"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="27">
         <v>151.62</v>
       </c>
-      <c r="D4" s="24">
+      <c r="D4" s="27">
         <v>187.3</v>
       </c>
-      <c r="E4" s="24">
+      <c r="E4" s="27">
         <v>195.27</v>
       </c>
-      <c r="F4" s="24">
+      <c r="F4" s="27">
         <v>206.45</v>
       </c>
-      <c r="G4" s="24">
+      <c r="G4" s="27">
         <v>214.07</v>
       </c>
       <c r="N4" s="3" t="s">
@@ -1441,14 +1469,14 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A5" s="20"/>
-      <c r="B5" s="21"/>
-      <c r="C5" s="24"/>
-      <c r="D5" s="24"/>
-      <c r="E5" s="24"/>
-      <c r="F5" s="24"/>
-      <c r="G5" s="24"/>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A5" s="23"/>
+      <c r="B5" s="24"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="27"/>
       <c r="N5" s="3" t="s">
         <v>30</v>
       </c>
@@ -1471,7 +1499,7 @@
         <v>31.161112290000002</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B6" s="7" t="s">
         <v>19</v>
       </c>
@@ -1516,7 +1544,7 @@
         <v>0.29092152256564102</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B7" s="7" t="s">
         <v>24</v>
       </c>
@@ -1559,7 +1587,7 @@
         <v>5.708245328833919</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B8" s="7" t="s">
         <v>25</v>
       </c>
@@ -1602,7 +1630,7 @@
         <v>30.870190767434362</v>
       </c>
     </row>
-    <row r="9" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>26</v>
       </c>
@@ -1644,16 +1672,16 @@
         <v>28.646099032989916</v>
       </c>
     </row>
-    <row r="10" spans="1:20" ht="18" x14ac:dyDescent="0.35">
-      <c r="A10" s="13" t="s">
+    <row r="10" spans="1:20" ht="15.6" x14ac:dyDescent="0.35">
+      <c r="A10" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="14"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="15"/>
+      <c r="B10" s="17"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="18"/>
       <c r="N10" s="3" t="s">
         <v>35</v>
       </c>
@@ -1676,18 +1704,18 @@
         <v>26.42200729854547</v>
       </c>
     </row>
-    <row r="11" spans="1:20" ht="18" x14ac:dyDescent="0.35">
-      <c r="A11" s="16" t="s">
+    <row r="11" spans="1:20" ht="15.6" x14ac:dyDescent="0.35">
+      <c r="A11" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="17"/>
-      <c r="C11" s="22" t="s">
+      <c r="B11" s="20"/>
+      <c r="C11" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="D11" s="22"/>
-      <c r="E11" s="22"/>
-      <c r="F11" s="22"/>
-      <c r="G11" s="23"/>
+      <c r="D11" s="25"/>
+      <c r="E11" s="25"/>
+      <c r="F11" s="25"/>
+      <c r="G11" s="26"/>
       <c r="N11" s="3" t="s">
         <v>36</v>
       </c>
@@ -1710,9 +1738,9 @@
         <v>0.98994638988464256</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A12" s="18"/>
-      <c r="B12" s="19"/>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A12" s="21"/>
+      <c r="B12" s="22"/>
       <c r="C12" s="1" t="s">
         <v>6</v>
       </c>
@@ -1750,22 +1778,22 @@
         <v>4.6709789600000002</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A13" s="18"/>
-      <c r="B13" s="19"/>
-      <c r="C13" s="24">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A13" s="21"/>
+      <c r="B13" s="22"/>
+      <c r="C13" s="27">
         <v>137.54</v>
       </c>
-      <c r="D13" s="24">
+      <c r="D13" s="27">
         <v>165.75</v>
       </c>
-      <c r="E13" s="24">
+      <c r="E13" s="27">
         <v>172.9</v>
       </c>
-      <c r="F13" s="24">
+      <c r="F13" s="27">
         <v>179.8</v>
       </c>
-      <c r="G13" s="24">
+      <c r="G13" s="27">
         <v>183.9</v>
       </c>
       <c r="N13" s="3" t="s">
@@ -1790,14 +1818,14 @@
         <v>8.5676397800000004</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A14" s="20"/>
-      <c r="B14" s="21"/>
-      <c r="C14" s="24"/>
-      <c r="D14" s="24"/>
-      <c r="E14" s="24"/>
-      <c r="F14" s="24"/>
-      <c r="G14" s="24"/>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A14" s="23"/>
+      <c r="B14" s="24"/>
+      <c r="C14" s="27"/>
+      <c r="D14" s="27"/>
+      <c r="E14" s="27"/>
+      <c r="F14" s="27"/>
+      <c r="G14" s="27"/>
       <c r="N14" s="3" t="s">
         <v>39</v>
       </c>
@@ -1820,7 +1848,7 @@
         <v>24.178772760488858</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A15" s="10"/>
       <c r="B15" s="7" t="s">
         <v>19</v>
@@ -1866,7 +1894,7 @@
         <v>4.2357627200000003</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B16" s="7" t="s">
         <v>24</v>
       </c>
@@ -1909,7 +1937,7 @@
         <v>7.0940057399999992</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B17" s="7" t="s">
         <v>25</v>
       </c>
@@ -1952,7 +1980,7 @@
         <v>0.36178175000000001</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
         <v>26</v>
       </c>
@@ -1994,7 +2022,7 @@
         <v>54.302358825637938</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N19" s="3" t="s">
         <v>44</v>
       </c>
@@ -2017,7 +2045,7 @@
         <v>1.1158962699999997</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N20" s="3" t="s">
         <v>45</v>
       </c>
@@ -2040,7 +2068,7 @@
         <v>40368.159200000002</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>20</v>
       </c>
@@ -2072,7 +2100,7 @@
         <v>-16.189386439511143</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>21</v>
       </c>
@@ -2098,7 +2126,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
         <v>12</v>
       </c>
@@ -2138,7 +2166,7 @@
         <v>0.75061547957059027</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
         <v>13</v>
       </c>
@@ -2171,7 +2199,7 @@
         <v>7456.9033862699989</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A25" s="7" t="s">
         <v>17</v>
       </c>
@@ -2208,7 +2236,7 @@
         <v>67.099101114943267</v>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
         <v>18</v>
       </c>
@@ -2245,7 +2273,7 @@
         <v>8.3779786486448486</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A27" s="8" t="s">
         <v>23</v>
       </c>
@@ -2278,7 +2306,7 @@
         <v>3652.0872323173585</v>
       </c>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
         <v>18</v>
       </c>
@@ -2297,7 +2325,7 @@
       <c r="S28" s="3"/>
       <c r="T28" s="3"/>
     </row>
-    <row r="29" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="8" t="s">
         <v>22</v>
       </c>
@@ -2318,7 +2346,7 @@
       <c r="S29" s="11"/>
       <c r="T29" s="11"/>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N30" s="3"/>
       <c r="O30" s="3" t="s">
         <v>27</v>
@@ -2339,7 +2367,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N31" s="3" t="s">
         <v>28</v>
       </c>
@@ -2362,7 +2390,7 @@
         <v>1799.9672083200001</v>
       </c>
     </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A32" s="7" t="s">
         <v>54</v>
       </c>
@@ -2395,7 +2423,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A33" s="7" t="s">
         <v>55</v>
       </c>
@@ -2428,7 +2456,7 @@
         <v>18.706244290000001</v>
       </c>
     </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A34" s="7" t="s">
         <v>56</v>
       </c>
@@ -2461,7 +2489,7 @@
         <v>0.17574765294122172</v>
       </c>
     </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N35" s="3" t="s">
         <v>32</v>
       </c>
@@ -2484,7 +2512,7 @@
         <v>3.4278460399999999</v>
       </c>
     </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N36" s="3" t="s">
         <v>33</v>
       </c>
@@ -2507,7 +2535,7 @@
         <v>18.530496637058778</v>
       </c>
     </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N37" s="3" t="s">
         <v>34</v>
       </c>
@@ -2530,7 +2558,7 @@
         <v>17.185376043221318</v>
       </c>
     </row>
-    <row r="38" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N38" s="3" t="s">
         <v>35</v>
       </c>
@@ -2553,7 +2581,7 @@
         <v>15.840255449383857</v>
       </c>
     </row>
-    <row r="39" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N39" s="3" t="s">
         <v>36</v>
       </c>
@@ -2576,7 +2604,7 @@
         <v>0.98987694252877945</v>
       </c>
     </row>
-    <row r="40" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N40" s="3" t="s">
         <v>37</v>
       </c>
@@ -2599,7 +2627,7 @@
         <v>2.8013522599999998</v>
       </c>
     </row>
-    <row r="41" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N41" s="3" t="s">
         <v>38</v>
       </c>
@@ -2622,7 +2650,7 @@
         <v>5.1205206399999996</v>
       </c>
     </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N42" s="3" t="s">
         <v>39</v>
       </c>
@@ -2645,7 +2673,7 @@
         <v>14.573233709896117</v>
       </c>
     </row>
-    <row r="43" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N43" s="3" t="s">
         <v>40</v>
       </c>
@@ -2668,7 +2696,7 @@
         <v>4.2514259799999996</v>
       </c>
     </row>
-    <row r="44" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N44" s="3" t="s">
         <v>41</v>
       </c>
@@ -2691,7 +2719,7 @@
         <v>4.2397910899999998</v>
       </c>
     </row>
-    <row r="45" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N45" s="3" t="s">
         <v>42</v>
       </c>
@@ -2714,7 +2742,7 @@
         <v>0.18547881599999999</v>
       </c>
     </row>
-    <row r="46" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N46" s="3" t="s">
         <v>43</v>
       </c>
@@ -2737,7 +2765,7 @@
         <v>54.474585290604679</v>
       </c>
     </row>
-    <row r="47" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N47" s="3" t="s">
         <v>44</v>
       </c>
@@ -2760,7 +2788,7 @@
         <v>0.67222976928854927</v>
       </c>
     </row>
-    <row r="48" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N48" s="3" t="s">
         <v>45</v>
       </c>
@@ -2783,7 +2811,7 @@
         <v>23737.731500000002</v>
       </c>
     </row>
-    <row r="49" spans="14:20" x14ac:dyDescent="0.25">
+    <row r="49" spans="14:20" x14ac:dyDescent="0.3">
       <c r="N49" s="3" t="s">
         <v>46</v>
       </c>
@@ -2806,7 +2834,7 @@
         <v>-9.1644977901038853</v>
       </c>
     </row>
-    <row r="50" spans="14:20" x14ac:dyDescent="0.25">
+    <row r="50" spans="14:20" x14ac:dyDescent="0.3">
       <c r="N50" s="3"/>
       <c r="O50" s="12"/>
       <c r="P50" s="12"/>
@@ -2823,7 +2851,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="14:20" x14ac:dyDescent="0.25">
+    <row r="51" spans="14:20" x14ac:dyDescent="0.3">
       <c r="N51" s="3" t="s">
         <v>51</v>
       </c>
@@ -2846,7 +2874,7 @@
         <v>0.74863011783778244</v>
       </c>
     </row>
-    <row r="52" spans="14:20" x14ac:dyDescent="0.25">
+    <row r="52" spans="14:20" x14ac:dyDescent="0.3">
       <c r="N52" s="3" t="s">
         <v>47</v>
       </c>
@@ -2869,7 +2897,7 @@
         <v>4425.9421357692881</v>
       </c>
     </row>
-    <row r="53" spans="14:20" x14ac:dyDescent="0.25">
+    <row r="53" spans="14:20" x14ac:dyDescent="0.3">
       <c r="N53" s="3" t="s">
         <v>52</v>
       </c>
@@ -2892,7 +2920,7 @@
         <v>66.346218081835687</v>
       </c>
     </row>
-    <row r="54" spans="14:20" x14ac:dyDescent="0.25">
+    <row r="54" spans="14:20" x14ac:dyDescent="0.3">
       <c r="N54" s="3" t="s">
         <v>48</v>
       </c>
@@ -2915,7 +2943,7 @@
         <v>8.4360410255996303</v>
       </c>
     </row>
-    <row r="55" spans="14:20" x14ac:dyDescent="0.25">
+    <row r="55" spans="14:20" x14ac:dyDescent="0.3">
       <c r="N55" s="3" t="s">
         <v>49</v>
       </c>
@@ -2940,6 +2968,14 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:B5"/>
+    <mergeCell ref="C2:G2"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="F4:F5"/>
+    <mergeCell ref="G4:G5"/>
     <mergeCell ref="A10:G10"/>
     <mergeCell ref="A11:B14"/>
     <mergeCell ref="C11:G11"/>
@@ -2948,14 +2984,6 @@
     <mergeCell ref="E13:E14"/>
     <mergeCell ref="F13:F14"/>
     <mergeCell ref="G13:G14"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:B5"/>
-    <mergeCell ref="C2:G2"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="F4:F5"/>
-    <mergeCell ref="G4:G5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated all technology cost and performance for cement (Cal was fine)
</commit_message>
<xml_diff>
--- a/adopt_net0/database/templates/technology_data/Industrial/CementHybridCCS_data/cement_sheet.xlsx
+++ b/adopt_net0/database/templates/technology_data/Industrial/CementHybridCCS_data/cement_sheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\AdOpT-NET0\adopt_net0\database\templates\technology_data\Industrial\CementHybridCCS_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\0954659\PycharmProjects\AdOpT-NET0_luca\adopt_net0\database\templates\technology_data\Industrial\CementHybridCCS_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C1A2A18-7943-4B3D-9E3F-F96EF1E288A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{658DCB68-ED6F-4AAF-8F21-D5C874F275B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-4404" windowWidth="30936" windowHeight="16896" activeTab="2" xr2:uid="{C0ECAA26-0769-408D-9398-31AECF4E3649}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{C0ECAA26-0769-408D-9398-31AECF4E3649}"/>
   </bookViews>
   <sheets>
     <sheet name="capex_oxyfuel" sheetId="1" r:id="rId1"/>
@@ -41,6 +41,41 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Bertoni, L. (Luca)</author>
+  </authors>
+  <commentList>
+    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{7B92FD06-FE8D-4C61-9A23-3AA36E43FCFA}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Bertoni, L. (Luca):</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+In euro totali
+</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="68">
   <si>
@@ -324,7 +359,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -383,6 +418,19 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -968,15 +1016,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D08EB36-8885-41F7-B3E9-60083815A79B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D08EB36-8885-41F7-B3E9-60083815A79B}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -984,7 +1032,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>75</v>
       </c>
@@ -992,7 +1040,7 @@
         <v>137540000</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>125</v>
       </c>
@@ -1002,19 +1050,20 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{447E0F8A-1C59-405C-B3D0-EB533A2330E6}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -1022,7 +1071,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <f>calculations!D15</f>
         <v>3.7084942228242932</v>
@@ -1032,7 +1081,7 @@
         <v>28210000.000000007</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <f>calculations!G15</f>
         <v>12.361647409414312</v>
@@ -1042,7 +1091,7 @@
         <v>46360000.000000015</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <f>calculations!G6</f>
         <v>20.602745682357188</v>
@@ -1061,9 +1110,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E17DFFB0-96B6-4F96-B3DF-E2D36B37C43F}">
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -1077,7 +1126,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0</v>
       </c>
@@ -1091,7 +1140,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>75</v>
       </c>
@@ -1105,7 +1154,7 @@
         <v>61000000</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>125</v>
       </c>
@@ -1127,15 +1176,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8995DE27-F5E7-40F1-8502-5CC793EB5921}">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -1149,7 +1198,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0</v>
       </c>
@@ -1163,7 +1212,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3">
         <f>calculations!D15</f>
         <v>3.7084942228242932</v>
@@ -1180,7 +1229,7 @@
         <v>10684945.673991</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4">
         <f>calculations!G15</f>
         <v>12.361647409414312</v>
@@ -1198,7 +1247,7 @@
         <v>16588739.769484399</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5">
         <f>calculations!G6</f>
         <v>20.602745682357188</v>
@@ -1224,14 +1273,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69712579-C7D8-42EE-9801-1FD637D0A17F}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>58</v>
       </c>
@@ -1240,7 +1289,7 @@
         <v>0.25548249251013122</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>59</v>
       </c>
@@ -1249,7 +1298,7 @@
         <v>8.2307186539958971E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>60</v>
       </c>
@@ -1266,12 +1315,12 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21185F42-04E5-4941-B133-36036095D1EF}">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>63</v>
       </c>
@@ -1285,7 +1334,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>62</v>
       </c>
@@ -1300,7 +1349,7 @@
       </c>
       <c r="E2" s="13"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>67</v>
       </c>
@@ -1315,7 +1364,7 @@
       </c>
       <c r="E3" s="13"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="13"/>
       <c r="B4" s="13"/>
       <c r="C4" s="13"/>
@@ -1330,14 +1379,14 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB78D47C-565F-4352-814A-A37F11C35FBF}">
   <dimension ref="A1:T55"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="52" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="16.2" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:20" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="16" t="s">
         <v>3</v>
       </c>
@@ -1357,7 +1406,7 @@
       <c r="S1" s="11"/>
       <c r="T1" s="3"/>
     </row>
-    <row r="2" spans="1:20" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:20" ht="18" x14ac:dyDescent="0.35">
       <c r="A2" s="19" t="s">
         <v>4</v>
       </c>
@@ -1389,7 +1438,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="21"/>
       <c r="B3" s="22"/>
       <c r="C3" s="1" t="s">
@@ -1429,7 +1478,7 @@
         <v>3000.20095584</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="21"/>
       <c r="B4" s="22"/>
       <c r="C4" s="27">
@@ -1469,7 +1518,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="23"/>
       <c r="B5" s="24"/>
       <c r="C5" s="27"/>
@@ -1499,7 +1548,7 @@
         <v>31.161112290000002</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B6" s="7" t="s">
         <v>19</v>
       </c>
@@ -1544,7 +1593,7 @@
         <v>0.29092152256564102</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B7" s="7" t="s">
         <v>24</v>
       </c>
@@ -1587,7 +1636,7 @@
         <v>5.708245328833919</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B8" s="7" t="s">
         <v>25</v>
       </c>
@@ -1630,7 +1679,7 @@
         <v>30.870190767434362</v>
       </c>
     </row>
-    <row r="9" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>26</v>
       </c>
@@ -1672,7 +1721,7 @@
         <v>28.646099032989916</v>
       </c>
     </row>
-    <row r="10" spans="1:20" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:20" ht="18" x14ac:dyDescent="0.35">
       <c r="A10" s="16" t="s">
         <v>11</v>
       </c>
@@ -1704,7 +1753,7 @@
         <v>26.42200729854547</v>
       </c>
     </row>
-    <row r="11" spans="1:20" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:20" ht="18" x14ac:dyDescent="0.35">
       <c r="A11" s="19" t="s">
         <v>4</v>
       </c>
@@ -1738,7 +1787,7 @@
         <v>0.98994638988464256</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" s="21"/>
       <c r="B12" s="22"/>
       <c r="C12" s="1" t="s">
@@ -1778,7 +1827,7 @@
         <v>4.6709789600000002</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A13" s="21"/>
       <c r="B13" s="22"/>
       <c r="C13" s="27">
@@ -1818,7 +1867,7 @@
         <v>8.5676397800000004</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14" s="23"/>
       <c r="B14" s="24"/>
       <c r="C14" s="27"/>
@@ -1848,7 +1897,7 @@
         <v>24.178772760488858</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15" s="10"/>
       <c r="B15" s="7" t="s">
         <v>19</v>
@@ -1894,7 +1943,7 @@
         <v>4.2357627200000003</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B16" s="7" t="s">
         <v>24</v>
       </c>
@@ -1937,7 +1986,7 @@
         <v>7.0940057399999992</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B17" s="7" t="s">
         <v>25</v>
       </c>
@@ -1980,7 +2029,7 @@
         <v>0.36178175000000001</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>26</v>
       </c>
@@ -2022,7 +2071,7 @@
         <v>54.302358825637938</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N19" s="3" t="s">
         <v>44</v>
       </c>
@@ -2045,7 +2094,7 @@
         <v>1.1158962699999997</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N20" s="3" t="s">
         <v>45</v>
       </c>
@@ -2068,7 +2117,7 @@
         <v>40368.159200000002</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>20</v>
       </c>
@@ -2100,7 +2149,7 @@
         <v>-16.189386439511143</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
         <v>21</v>
       </c>
@@ -2126,7 +2175,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
         <v>12</v>
       </c>
@@ -2166,7 +2215,7 @@
         <v>0.75061547957059027</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
         <v>13</v>
       </c>
@@ -2199,7 +2248,7 @@
         <v>7456.9033862699989</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
         <v>17</v>
       </c>
@@ -2236,7 +2285,7 @@
         <v>67.099101114943267</v>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>18</v>
       </c>
@@ -2273,7 +2322,7 @@
         <v>8.3779786486448486</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
         <v>23</v>
       </c>
@@ -2306,7 +2355,7 @@
         <v>3652.0872323173585</v>
       </c>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
         <v>18</v>
       </c>
@@ -2325,7 +2374,7 @@
       <c r="S28" s="3"/>
       <c r="T28" s="3"/>
     </row>
-    <row r="29" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="8" t="s">
         <v>22</v>
       </c>
@@ -2346,7 +2395,7 @@
       <c r="S29" s="11"/>
       <c r="T29" s="11"/>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N30" s="3"/>
       <c r="O30" s="3" t="s">
         <v>27</v>
@@ -2367,7 +2416,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N31" s="3" t="s">
         <v>28</v>
       </c>
@@ -2390,7 +2439,7 @@
         <v>1799.9672083200001</v>
       </c>
     </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A32" s="7" t="s">
         <v>54</v>
       </c>
@@ -2423,7 +2472,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
         <v>55</v>
       </c>
@@ -2456,7 +2505,7 @@
         <v>18.706244290000001</v>
       </c>
     </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A34" s="7" t="s">
         <v>56</v>
       </c>
@@ -2489,7 +2538,7 @@
         <v>0.17574765294122172</v>
       </c>
     </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N35" s="3" t="s">
         <v>32</v>
       </c>
@@ -2512,7 +2561,7 @@
         <v>3.4278460399999999</v>
       </c>
     </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N36" s="3" t="s">
         <v>33</v>
       </c>
@@ -2535,7 +2584,7 @@
         <v>18.530496637058778</v>
       </c>
     </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N37" s="3" t="s">
         <v>34</v>
       </c>
@@ -2558,7 +2607,7 @@
         <v>17.185376043221318</v>
       </c>
     </row>
-    <row r="38" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N38" s="3" t="s">
         <v>35</v>
       </c>
@@ -2581,7 +2630,7 @@
         <v>15.840255449383857</v>
       </c>
     </row>
-    <row r="39" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N39" s="3" t="s">
         <v>36</v>
       </c>
@@ -2604,7 +2653,7 @@
         <v>0.98987694252877945</v>
       </c>
     </row>
-    <row r="40" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N40" s="3" t="s">
         <v>37</v>
       </c>
@@ -2627,7 +2676,7 @@
         <v>2.8013522599999998</v>
       </c>
     </row>
-    <row r="41" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N41" s="3" t="s">
         <v>38</v>
       </c>
@@ -2650,7 +2699,7 @@
         <v>5.1205206399999996</v>
       </c>
     </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N42" s="3" t="s">
         <v>39</v>
       </c>
@@ -2673,7 +2722,7 @@
         <v>14.573233709896117</v>
       </c>
     </row>
-    <row r="43" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N43" s="3" t="s">
         <v>40</v>
       </c>
@@ -2696,7 +2745,7 @@
         <v>4.2514259799999996</v>
       </c>
     </row>
-    <row r="44" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N44" s="3" t="s">
         <v>41</v>
       </c>
@@ -2719,7 +2768,7 @@
         <v>4.2397910899999998</v>
       </c>
     </row>
-    <row r="45" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N45" s="3" t="s">
         <v>42</v>
       </c>
@@ -2742,7 +2791,7 @@
         <v>0.18547881599999999</v>
       </c>
     </row>
-    <row r="46" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N46" s="3" t="s">
         <v>43</v>
       </c>
@@ -2765,7 +2814,7 @@
         <v>54.474585290604679</v>
       </c>
     </row>
-    <row r="47" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N47" s="3" t="s">
         <v>44</v>
       </c>
@@ -2788,7 +2837,7 @@
         <v>0.67222976928854927</v>
       </c>
     </row>
-    <row r="48" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N48" s="3" t="s">
         <v>45</v>
       </c>
@@ -2811,7 +2860,7 @@
         <v>23737.731500000002</v>
       </c>
     </row>
-    <row r="49" spans="14:20" x14ac:dyDescent="0.3">
+    <row r="49" spans="14:20" x14ac:dyDescent="0.25">
       <c r="N49" s="3" t="s">
         <v>46</v>
       </c>
@@ -2834,7 +2883,7 @@
         <v>-9.1644977901038853</v>
       </c>
     </row>
-    <row r="50" spans="14:20" x14ac:dyDescent="0.3">
+    <row r="50" spans="14:20" x14ac:dyDescent="0.25">
       <c r="N50" s="3"/>
       <c r="O50" s="12"/>
       <c r="P50" s="12"/>
@@ -2851,7 +2900,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="14:20" x14ac:dyDescent="0.3">
+    <row r="51" spans="14:20" x14ac:dyDescent="0.25">
       <c r="N51" s="3" t="s">
         <v>51</v>
       </c>
@@ -2874,7 +2923,7 @@
         <v>0.74863011783778244</v>
       </c>
     </row>
-    <row r="52" spans="14:20" x14ac:dyDescent="0.3">
+    <row r="52" spans="14:20" x14ac:dyDescent="0.25">
       <c r="N52" s="3" t="s">
         <v>47</v>
       </c>
@@ -2897,7 +2946,7 @@
         <v>4425.9421357692881</v>
       </c>
     </row>
-    <row r="53" spans="14:20" x14ac:dyDescent="0.3">
+    <row r="53" spans="14:20" x14ac:dyDescent="0.25">
       <c r="N53" s="3" t="s">
         <v>52</v>
       </c>
@@ -2920,7 +2969,7 @@
         <v>66.346218081835687</v>
       </c>
     </row>
-    <row r="54" spans="14:20" x14ac:dyDescent="0.3">
+    <row r="54" spans="14:20" x14ac:dyDescent="0.25">
       <c r="N54" s="3" t="s">
         <v>48</v>
       </c>
@@ -2943,7 +2992,7 @@
         <v>8.4360410255996303</v>
       </c>
     </row>
-    <row r="55" spans="14:20" x14ac:dyDescent="0.3">
+    <row r="55" spans="14:20" x14ac:dyDescent="0.25">
       <c r="N55" s="3" t="s">
         <v>49</v>
       </c>
@@ -2968,6 +3017,14 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A10:G10"/>
+    <mergeCell ref="A11:B14"/>
+    <mergeCell ref="C11:G11"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="G13:G14"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:B5"/>
     <mergeCell ref="C2:G2"/>
@@ -2976,14 +3033,6 @@
     <mergeCell ref="E4:E5"/>
     <mergeCell ref="F4:F5"/>
     <mergeCell ref="G4:G5"/>
-    <mergeCell ref="A10:G10"/>
-    <mergeCell ref="A11:B14"/>
-    <mergeCell ref="C11:G11"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="F13:F14"/>
-    <mergeCell ref="G13:G14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Fixed bug on piecewise values for CementHybridCCS.json (capex non_zero at zero size)
</commit_message>
<xml_diff>
--- a/adopt_net0/database/templates/technology_data/Industrial/CementHybridCCS_data/cement_sheet.xlsx
+++ b/adopt_net0/database/templates/technology_data/Industrial/CementHybridCCS_data/cement_sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\0954659\PycharmProjects\AdOpT-NET0_luca\adopt_net0\database\templates\technology_data\Industrial\CementHybridCCS_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{658DCB68-ED6F-4AAF-8F21-D5C874F275B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75A02427-DF3E-4354-8547-86A55ED0E5EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{C0ECAA26-0769-408D-9398-31AECF4E3649}"/>
+    <workbookView xWindow="-30" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{C0ECAA26-0769-408D-9398-31AECF4E3649}"/>
   </bookViews>
   <sheets>
     <sheet name="capex_oxyfuel" sheetId="1" r:id="rId1"/>
@@ -1018,13 +1018,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D08EB36-8885-41F7-B3E9-60083815A79B}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1032,7 +1032,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>75</v>
       </c>
@@ -1040,7 +1040,7 @@
         <v>137540000</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>125</v>
       </c>
@@ -1057,13 +1057,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{447E0F8A-1C59-405C-B3D0-EB533A2330E6}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -1071,7 +1071,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2">
         <f>calculations!D15</f>
         <v>3.7084942228242932</v>
@@ -1081,7 +1081,7 @@
         <v>28210000.000000007</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3">
         <f>calculations!G15</f>
         <v>12.361647409414312</v>
@@ -1091,7 +1091,7 @@
         <v>46360000.000000015</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4">
         <f>calculations!G6</f>
         <v>20.602745682357188</v>
@@ -1110,9 +1110,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E17DFFB0-96B6-4F96-B3DF-E2D36B37C43F}">
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -1126,7 +1126,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>0</v>
       </c>
@@ -1140,7 +1140,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>75</v>
       </c>
@@ -1154,7 +1154,7 @@
         <v>61000000</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>125</v>
       </c>
@@ -1176,15 +1176,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8995DE27-F5E7-40F1-8502-5CC793EB5921}">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -1198,7 +1198,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>0</v>
       </c>
@@ -1212,7 +1212,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3">
         <f>calculations!D15</f>
         <v>3.7084942228242932</v>
@@ -1229,7 +1229,7 @@
         <v>10684945.673991</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4">
         <f>calculations!G15</f>
         <v>12.361647409414312</v>
@@ -1247,7 +1247,7 @@
         <v>16588739.769484399</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5">
         <f>calculations!G6</f>
         <v>20.602745682357188</v>
@@ -1273,14 +1273,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69712579-C7D8-42EE-9801-1FD637D0A17F}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>58</v>
       </c>
@@ -1289,7 +1289,7 @@
         <v>0.25548249251013122</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>59</v>
       </c>
@@ -1298,7 +1298,7 @@
         <v>8.2307186539958971E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>60</v>
       </c>
@@ -1315,12 +1315,12 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21185F42-04E5-4941-B133-36036095D1EF}">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>63</v>
       </c>
@@ -1334,7 +1334,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="13" t="s">
         <v>62</v>
       </c>
@@ -1349,7 +1349,7 @@
       </c>
       <c r="E2" s="13"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="13" t="s">
         <v>67</v>
       </c>
@@ -1364,7 +1364,7 @@
       </c>
       <c r="E3" s="13"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="13"/>
       <c r="B4" s="13"/>
       <c r="C4" s="13"/>
@@ -1379,14 +1379,14 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB78D47C-565F-4352-814A-A37F11C35FBF}">
   <dimension ref="A1:T55"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="52" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:20" ht="16.2" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="16" t="s">
         <v>3</v>
       </c>
@@ -1406,7 +1406,7 @@
       <c r="S1" s="11"/>
       <c r="T1" s="3"/>
     </row>
-    <row r="2" spans="1:20" ht="18" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:20" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A2" s="19" t="s">
         <v>4</v>
       </c>
@@ -1438,7 +1438,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A3" s="21"/>
       <c r="B3" s="22"/>
       <c r="C3" s="1" t="s">
@@ -1478,7 +1478,7 @@
         <v>3000.20095584</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A4" s="21"/>
       <c r="B4" s="22"/>
       <c r="C4" s="27">
@@ -1518,7 +1518,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A5" s="23"/>
       <c r="B5" s="24"/>
       <c r="C5" s="27"/>
@@ -1548,7 +1548,7 @@
         <v>31.161112290000002</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B6" s="7" t="s">
         <v>19</v>
       </c>
@@ -1593,7 +1593,7 @@
         <v>0.29092152256564102</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B7" s="7" t="s">
         <v>24</v>
       </c>
@@ -1636,7 +1636,7 @@
         <v>5.708245328833919</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B8" s="7" t="s">
         <v>25</v>
       </c>
@@ -1679,7 +1679,7 @@
         <v>30.870190767434362</v>
       </c>
     </row>
-    <row r="9" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>26</v>
       </c>
@@ -1721,7 +1721,7 @@
         <v>28.646099032989916</v>
       </c>
     </row>
-    <row r="10" spans="1:20" ht="18" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:20" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A10" s="16" t="s">
         <v>11</v>
       </c>
@@ -1753,7 +1753,7 @@
         <v>26.42200729854547</v>
       </c>
     </row>
-    <row r="11" spans="1:20" ht="18" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:20" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A11" s="19" t="s">
         <v>4</v>
       </c>
@@ -1787,7 +1787,7 @@
         <v>0.98994638988464256</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A12" s="21"/>
       <c r="B12" s="22"/>
       <c r="C12" s="1" t="s">
@@ -1827,7 +1827,7 @@
         <v>4.6709789600000002</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A13" s="21"/>
       <c r="B13" s="22"/>
       <c r="C13" s="27">
@@ -1867,7 +1867,7 @@
         <v>8.5676397800000004</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A14" s="23"/>
       <c r="B14" s="24"/>
       <c r="C14" s="27"/>
@@ -1897,7 +1897,7 @@
         <v>24.178772760488858</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A15" s="10"/>
       <c r="B15" s="7" t="s">
         <v>19</v>
@@ -1943,7 +1943,7 @@
         <v>4.2357627200000003</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B16" s="7" t="s">
         <v>24</v>
       </c>
@@ -1986,7 +1986,7 @@
         <v>7.0940057399999992</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B17" s="7" t="s">
         <v>25</v>
       </c>
@@ -2029,7 +2029,7 @@
         <v>0.36178175000000001</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
         <v>26</v>
       </c>
@@ -2071,7 +2071,7 @@
         <v>54.302358825637938</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N19" s="3" t="s">
         <v>44</v>
       </c>
@@ -2094,7 +2094,7 @@
         <v>1.1158962699999997</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N20" s="3" t="s">
         <v>45</v>
       </c>
@@ -2117,7 +2117,7 @@
         <v>40368.159200000002</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>20</v>
       </c>
@@ -2149,7 +2149,7 @@
         <v>-16.189386439511143</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>21</v>
       </c>
@@ -2175,7 +2175,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
         <v>12</v>
       </c>
@@ -2215,7 +2215,7 @@
         <v>0.75061547957059027</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
         <v>13</v>
       </c>
@@ -2248,7 +2248,7 @@
         <v>7456.9033862699989</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A25" s="7" t="s">
         <v>17</v>
       </c>
@@ -2285,7 +2285,7 @@
         <v>67.099101114943267</v>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
         <v>18</v>
       </c>
@@ -2322,7 +2322,7 @@
         <v>8.3779786486448486</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A27" s="8" t="s">
         <v>23</v>
       </c>
@@ -2355,7 +2355,7 @@
         <v>3652.0872323173585</v>
       </c>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
         <v>18</v>
       </c>
@@ -2374,7 +2374,7 @@
       <c r="S28" s="3"/>
       <c r="T28" s="3"/>
     </row>
-    <row r="29" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="8" t="s">
         <v>22</v>
       </c>
@@ -2395,7 +2395,7 @@
       <c r="S29" s="11"/>
       <c r="T29" s="11"/>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N30" s="3"/>
       <c r="O30" s="3" t="s">
         <v>27</v>
@@ -2416,7 +2416,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N31" s="3" t="s">
         <v>28</v>
       </c>
@@ -2439,7 +2439,7 @@
         <v>1799.9672083200001</v>
       </c>
     </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A32" s="7" t="s">
         <v>54</v>
       </c>
@@ -2472,7 +2472,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A33" s="7" t="s">
         <v>55</v>
       </c>
@@ -2505,7 +2505,7 @@
         <v>18.706244290000001</v>
       </c>
     </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A34" s="7" t="s">
         <v>56</v>
       </c>
@@ -2538,7 +2538,7 @@
         <v>0.17574765294122172</v>
       </c>
     </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N35" s="3" t="s">
         <v>32</v>
       </c>
@@ -2561,7 +2561,7 @@
         <v>3.4278460399999999</v>
       </c>
     </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N36" s="3" t="s">
         <v>33</v>
       </c>
@@ -2584,7 +2584,7 @@
         <v>18.530496637058778</v>
       </c>
     </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N37" s="3" t="s">
         <v>34</v>
       </c>
@@ -2607,7 +2607,7 @@
         <v>17.185376043221318</v>
       </c>
     </row>
-    <row r="38" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N38" s="3" t="s">
         <v>35</v>
       </c>
@@ -2630,7 +2630,7 @@
         <v>15.840255449383857</v>
       </c>
     </row>
-    <row r="39" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N39" s="3" t="s">
         <v>36</v>
       </c>
@@ -2653,7 +2653,7 @@
         <v>0.98987694252877945</v>
       </c>
     </row>
-    <row r="40" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N40" s="3" t="s">
         <v>37</v>
       </c>
@@ -2676,7 +2676,7 @@
         <v>2.8013522599999998</v>
       </c>
     </row>
-    <row r="41" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N41" s="3" t="s">
         <v>38</v>
       </c>
@@ -2699,7 +2699,7 @@
         <v>5.1205206399999996</v>
       </c>
     </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N42" s="3" t="s">
         <v>39</v>
       </c>
@@ -2722,7 +2722,7 @@
         <v>14.573233709896117</v>
       </c>
     </row>
-    <row r="43" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N43" s="3" t="s">
         <v>40</v>
       </c>
@@ -2745,7 +2745,7 @@
         <v>4.2514259799999996</v>
       </c>
     </row>
-    <row r="44" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N44" s="3" t="s">
         <v>41</v>
       </c>
@@ -2768,7 +2768,7 @@
         <v>4.2397910899999998</v>
       </c>
     </row>
-    <row r="45" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N45" s="3" t="s">
         <v>42</v>
       </c>
@@ -2791,7 +2791,7 @@
         <v>0.18547881599999999</v>
       </c>
     </row>
-    <row r="46" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N46" s="3" t="s">
         <v>43</v>
       </c>
@@ -2814,7 +2814,7 @@
         <v>54.474585290604679</v>
       </c>
     </row>
-    <row r="47" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N47" s="3" t="s">
         <v>44</v>
       </c>
@@ -2837,7 +2837,7 @@
         <v>0.67222976928854927</v>
       </c>
     </row>
-    <row r="48" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N48" s="3" t="s">
         <v>45</v>
       </c>
@@ -2860,7 +2860,7 @@
         <v>23737.731500000002</v>
       </c>
     </row>
-    <row r="49" spans="14:20" x14ac:dyDescent="0.25">
+    <row r="49" spans="14:20" x14ac:dyDescent="0.3">
       <c r="N49" s="3" t="s">
         <v>46</v>
       </c>
@@ -2883,7 +2883,7 @@
         <v>-9.1644977901038853</v>
       </c>
     </row>
-    <row r="50" spans="14:20" x14ac:dyDescent="0.25">
+    <row r="50" spans="14:20" x14ac:dyDescent="0.3">
       <c r="N50" s="3"/>
       <c r="O50" s="12"/>
       <c r="P50" s="12"/>
@@ -2900,7 +2900,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="14:20" x14ac:dyDescent="0.25">
+    <row r="51" spans="14:20" x14ac:dyDescent="0.3">
       <c r="N51" s="3" t="s">
         <v>51</v>
       </c>
@@ -2923,7 +2923,7 @@
         <v>0.74863011783778244</v>
       </c>
     </row>
-    <row r="52" spans="14:20" x14ac:dyDescent="0.25">
+    <row r="52" spans="14:20" x14ac:dyDescent="0.3">
       <c r="N52" s="3" t="s">
         <v>47</v>
       </c>
@@ -2946,7 +2946,7 @@
         <v>4425.9421357692881</v>
       </c>
     </row>
-    <row r="53" spans="14:20" x14ac:dyDescent="0.25">
+    <row r="53" spans="14:20" x14ac:dyDescent="0.3">
       <c r="N53" s="3" t="s">
         <v>52</v>
       </c>
@@ -2969,7 +2969,7 @@
         <v>66.346218081835687</v>
       </c>
     </row>
-    <row r="54" spans="14:20" x14ac:dyDescent="0.25">
+    <row r="54" spans="14:20" x14ac:dyDescent="0.3">
       <c r="N54" s="3" t="s">
         <v>48</v>
       </c>
@@ -2992,7 +2992,7 @@
         <v>8.4360410255996303</v>
       </c>
     </row>
-    <row r="55" spans="14:20" x14ac:dyDescent="0.25">
+    <row r="55" spans="14:20" x14ac:dyDescent="0.3">
       <c r="N55" s="3" t="s">
         <v>49</v>
       </c>
@@ -3017,6 +3017,14 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:B5"/>
+    <mergeCell ref="C2:G2"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="F4:F5"/>
+    <mergeCell ref="G4:G5"/>
     <mergeCell ref="A10:G10"/>
     <mergeCell ref="A11:B14"/>
     <mergeCell ref="C11:G11"/>
@@ -3025,14 +3033,6 @@
     <mergeCell ref="E13:E14"/>
     <mergeCell ref="F13:F14"/>
     <mergeCell ref="G13:G14"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:B5"/>
-    <mergeCell ref="C2:G2"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="F4:F5"/>
-    <mergeCell ref="G4:G5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added el_recovery_oxy to cement_hybrid_ccs.py
</commit_message>
<xml_diff>
--- a/adopt_net0/database/templates/technology_data/Industrial/CementHybridCCS_data/cement_sheet.xlsx
+++ b/adopt_net0/database/templates/technology_data/Industrial/CementHybridCCS_data/cement_sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\0954659\PycharmProjects\AdOpT-NET0_luca\adopt_net0\database\templates\technology_data\Industrial\CementHybridCCS_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D18EF57D-E260-4DFB-823D-C1BDDC582C0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FAE1B19-950B-46D2-A8AD-6DB545E78BF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28935" yWindow="-135" windowWidth="29070" windowHeight="15750" activeTab="1" xr2:uid="{C0ECAA26-0769-408D-9398-31AECF4E3649}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="4" xr2:uid="{C0ECAA26-0769-408D-9398-31AECF4E3649}"/>
   </bookViews>
   <sheets>
     <sheet name="capex_oxyfuel" sheetId="1" r:id="rId1"/>
@@ -77,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="64">
   <si>
     <t>size_tclinker_per_h</t>
   </si>
@@ -332,6 +332,12 @@
   </si>
   <si>
     <t>fixed OPEX Fraction of capex</t>
+  </si>
+  <si>
+    <t>electricity_recovery_oxy</t>
+  </si>
+  <si>
+    <t>el_recovery_oxy</t>
   </si>
 </sst>
 </file>
@@ -614,7 +620,7 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -649,6 +655,7 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="4" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="13" xfId="4" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="13" xfId="4" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -685,7 +692,8 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="3" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="13" xfId="4" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="13" xfId="4" applyFont="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Calculation" xfId="5" builtinId="22"/>
@@ -1026,13 +1034,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D08EB36-8885-41F7-B3E9-60083815A79B}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1040,7 +1048,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>75</v>
       </c>
@@ -1048,7 +1056,7 @@
         <v>50760000</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>125</v>
       </c>
@@ -1065,13 +1073,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{447E0F8A-1C59-405C-B3D0-EB533A2330E6}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -1079,7 +1087,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <f>calculations!D19</f>
         <v>4.4302472880300003</v>
@@ -1089,7 +1097,7 @@
         <v>13962331.812465826</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
         <f>calculations!G19</f>
         <v>14.767490960100002</v>
@@ -1103,7 +1111,7 @@
         <v>1717285.6288532494</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
         <f>calculations!G6</f>
         <v>24.418823252400006</v>
@@ -1122,9 +1130,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E17DFFB0-96B6-4F96-B3DF-E2D36B37C43F}">
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -1138,7 +1146,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>0</v>
       </c>
@@ -1152,7 +1160,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>75</v>
       </c>
@@ -1166,7 +1174,7 @@
         <v>61000000</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>125</v>
       </c>
@@ -1188,15 +1196,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8995DE27-F5E7-40F1-8502-5CC793EB5921}">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -1210,7 +1218,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>0</v>
       </c>
@@ -1224,7 +1232,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3">
         <f>calculations!D19</f>
         <v>4.4302472880300003</v>
@@ -1241,7 +1249,7 @@
         <v>10684945.673991</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4">
         <f>calculations!G19</f>
         <v>14.767490960100002</v>
@@ -1259,7 +1267,7 @@
         <v>16588739.769484399</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5">
         <f>calculations!G6</f>
         <v>24.418823252400006</v>
@@ -1284,18 +1292,18 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69712579-C7D8-42EE-9801-1FD637D0A17F}">
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>48</v>
       </c>
@@ -1304,22 +1312,31 @@
         <v>0.3128088466592428</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>49</v>
       </c>
       <c r="B3">
         <f>calculations!C40</f>
-        <v>-2.803449415155216E-2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+        <v>7.833563329433206E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>50</v>
       </c>
       <c r="B4">
         <f>calculations!C41</f>
         <v>3.8587338925408297E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>63</v>
+      </c>
+      <c r="B5">
+        <f>calculations!C38</f>
+        <v>0.10637012744588423</v>
       </c>
     </row>
   </sheetData>
@@ -1329,13 +1346,13 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21185F42-04E5-4941-B133-36036095D1EF}">
-  <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>53</v>
       </c>
@@ -1349,7 +1366,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="13" t="s">
         <v>52</v>
       </c>
@@ -1364,7 +1381,7 @@
       </c>
       <c r="E2" s="13"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="13" t="s">
         <v>57</v>
       </c>
@@ -1379,12 +1396,18 @@
       </c>
       <c r="E3" s="13"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="13"/>
       <c r="B4" s="13"/>
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
       <c r="E4" s="13"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D6" s="35"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D7" s="35"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1394,24 +1417,25 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB78D47C-565F-4352-814A-A37F11C35FBF}">
   <dimension ref="A1:T57"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.85546875" customWidth="1"/>
+    <col min="1" max="1" width="26.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.88671875" customWidth="1"/>
+    <col min="3" max="3" width="12.5546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="52" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="22" t="s">
+    <row r="1" spans="1:20" ht="16.2" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="24"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="25"/>
       <c r="N1" s="11"/>
       <c r="O1" s="11" t="s">
         <v>40</v>
@@ -1422,18 +1446,18 @@
       <c r="S1" s="11"/>
       <c r="T1" s="3"/>
     </row>
-    <row r="2" spans="1:20" ht="18" x14ac:dyDescent="0.35">
-      <c r="A2" s="25" t="s">
+    <row r="2" spans="1:20" ht="15.6" x14ac:dyDescent="0.35">
+      <c r="A2" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="31" t="s">
+      <c r="B2" s="27"/>
+      <c r="C2" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="33"/>
       <c r="N2" s="3"/>
       <c r="O2" s="3" t="s">
         <v>17</v>
@@ -1454,9 +1478,9 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A3" s="27"/>
-      <c r="B3" s="28"/>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A3" s="28"/>
+      <c r="B3" s="29"/>
       <c r="C3" s="1" t="s">
         <v>6</v>
       </c>
@@ -1494,22 +1518,22 @@
         <v>2999.91944736</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A4" s="27"/>
-      <c r="B4" s="28"/>
-      <c r="C4" s="33">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A4" s="28"/>
+      <c r="B4" s="29"/>
+      <c r="C4" s="34">
         <v>72.349999999999994</v>
       </c>
-      <c r="D4" s="33">
+      <c r="D4" s="34">
         <v>84.320988516056687</v>
       </c>
-      <c r="E4" s="33">
+      <c r="E4" s="34">
         <v>89.206549352337717</v>
       </c>
-      <c r="F4" s="33">
+      <c r="F4" s="34">
         <v>95.445590190807295</v>
       </c>
-      <c r="G4" s="33">
+      <c r="G4" s="34">
         <v>99.17</v>
       </c>
       <c r="N4" s="3" t="s">
@@ -1534,14 +1558,14 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A5" s="29"/>
-      <c r="B5" s="30"/>
-      <c r="C5" s="33"/>
-      <c r="D5" s="33"/>
-      <c r="E5" s="33"/>
-      <c r="F5" s="33"/>
-      <c r="G5" s="33"/>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A5" s="30"/>
+      <c r="B5" s="31"/>
+      <c r="C5" s="34"/>
+      <c r="D5" s="34"/>
+      <c r="E5" s="34"/>
+      <c r="F5" s="34"/>
+      <c r="G5" s="34"/>
       <c r="L5">
         <f>1-P6/P5</f>
         <v>0.78184911505744248</v>
@@ -1568,7 +1592,7 @@
         <v>32.665832100000003</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B6" s="7" t="s">
         <v>13</v>
       </c>
@@ -1613,7 +1637,7 @@
         <v>0.343073721</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B7" s="7" t="s">
         <v>14</v>
       </c>
@@ -1623,7 +1647,7 @@
         <v>11970988.516056692</v>
       </c>
       <c r="E7" s="7">
-        <f t="shared" ref="E7:G7" si="1">(E4-$C$4)*10^6</f>
+        <f t="shared" ref="E7:F7" si="1">(E4-$C$4)*10^6</f>
         <v>16856549.352337722</v>
       </c>
       <c r="F7" s="7">
@@ -1656,7 +1680,7 @@
         <v>6.7830064590000019</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B8" s="7" t="s">
         <v>15</v>
       </c>
@@ -1699,7 +1723,7 @@
         <v>32.322758379</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>16</v>
       </c>
@@ -1741,7 +1765,7 @@
         <v>29.496494612333333</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B10" s="19" t="s">
         <v>59</v>
       </c>
@@ -1786,7 +1810,7 @@
         <v>26.670230845666659</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B11" s="19" t="s">
         <v>60</v>
       </c>
@@ -1832,7 +1856,7 @@
         <v>0.98850272506734771</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B12" s="19" t="s">
         <v>61</v>
       </c>
@@ -1878,7 +1902,7 @@
         <v>5.1419803699999997</v>
       </c>
     </row>
-    <row r="13" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="N13" s="3" t="s">
         <v>28</v>
       </c>
@@ -1901,16 +1925,16 @@
         <v>8.4990979400000004</v>
       </c>
     </row>
-    <row r="14" spans="1:20" ht="18" x14ac:dyDescent="0.35">
-      <c r="A14" s="22" t="s">
+    <row r="14" spans="1:20" ht="15.6" x14ac:dyDescent="0.35">
+      <c r="A14" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="23"/>
-      <c r="C14" s="23"/>
-      <c r="D14" s="23"/>
-      <c r="E14" s="23"/>
-      <c r="F14" s="23"/>
-      <c r="G14" s="24"/>
+      <c r="B14" s="24"/>
+      <c r="C14" s="24"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="24"/>
+      <c r="F14" s="24"/>
+      <c r="G14" s="25"/>
       <c r="N14" s="3" t="s">
         <v>29</v>
       </c>
@@ -1933,18 +1957,18 @@
         <v>24.018188706552724</v>
       </c>
     </row>
-    <row r="15" spans="1:20" ht="18" x14ac:dyDescent="0.35">
-      <c r="A15" s="25" t="s">
+    <row r="15" spans="1:20" ht="15.6" x14ac:dyDescent="0.35">
+      <c r="A15" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="B15" s="26"/>
-      <c r="C15" s="31" t="s">
+      <c r="B15" s="27"/>
+      <c r="C15" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="D15" s="31"/>
-      <c r="E15" s="31"/>
-      <c r="F15" s="31"/>
-      <c r="G15" s="32"/>
+      <c r="D15" s="32"/>
+      <c r="E15" s="32"/>
+      <c r="F15" s="32"/>
+      <c r="G15" s="33"/>
       <c r="N15" s="3" t="s">
         <v>30</v>
       </c>
@@ -1967,9 +1991,9 @@
         <v>3.5409355499999999</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A16" s="27"/>
-      <c r="B16" s="28"/>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A16" s="28"/>
+      <c r="B16" s="29"/>
       <c r="C16" s="1" t="s">
         <v>6</v>
       </c>
@@ -2007,22 +2031,22 @@
         <v>7.0372530900000001</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A17" s="27"/>
-      <c r="B17" s="28"/>
-      <c r="C17" s="33">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A17" s="28"/>
+      <c r="B17" s="29"/>
+      <c r="C17" s="34">
         <v>50.76</v>
       </c>
-      <c r="D17" s="33">
+      <c r="D17" s="34">
         <v>64.722331812465825</v>
       </c>
-      <c r="E17" s="33">
+      <c r="E17" s="34">
         <v>68.47234583745032</v>
       </c>
-      <c r="F17" s="33">
+      <c r="F17" s="34">
         <v>73.261251641870047</v>
       </c>
-      <c r="G17" s="33">
+      <c r="G17" s="34">
         <v>76.12</v>
       </c>
       <c r="N17" s="3" t="s">
@@ -2047,14 +2071,14 @@
         <v>0.16516841700000001</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A18" s="29"/>
-      <c r="B18" s="30"/>
-      <c r="C18" s="33"/>
-      <c r="D18" s="33"/>
-      <c r="E18" s="33"/>
-      <c r="F18" s="33"/>
-      <c r="G18" s="33"/>
+    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A18" s="30"/>
+      <c r="B18" s="31"/>
+      <c r="C18" s="34"/>
+      <c r="D18" s="34"/>
+      <c r="E18" s="34"/>
+      <c r="F18" s="34"/>
+      <c r="G18" s="34"/>
       <c r="N18" s="3" t="s">
         <v>33</v>
       </c>
@@ -2077,7 +2101,7 @@
         <v>38.587338925408297</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A19" s="10"/>
       <c r="B19" s="7" t="s">
         <v>13</v>
@@ -2093,7 +2117,7 @@
         <f t="shared" ref="E19:G19" si="5">R36*3600/1000</f>
         <v>7.3837454800500009</v>
       </c>
-      <c r="F19" s="34">
+      <c r="F19" s="22">
         <f>S36*3600/1000</f>
         <v>11.81399276808</v>
       </c>
@@ -2123,7 +2147,7 @@
         <v>0.9422574090000001</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B20" s="7" t="s">
         <v>14</v>
       </c>
@@ -2144,7 +2168,9 @@
         <f t="shared" si="6"/>
         <v>25360000.000000007</v>
       </c>
-      <c r="N20" s="3"/>
+      <c r="N20" s="18" t="s">
+        <v>58</v>
+      </c>
       <c r="O20" s="16" t="s">
         <v>12</v>
       </c>
@@ -2164,7 +2190,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B21" s="7" t="s">
         <v>15</v>
       </c>
@@ -2207,7 +2233,7 @@
         <v>34915.217199999999</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B22" t="s">
         <v>16</v>
       </c>
@@ -2249,7 +2275,7 @@
         <v>-10.897028493447277</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B23" s="19" t="s">
         <v>59</v>
       </c>
@@ -2288,7 +2314,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B24" s="19" t="s">
         <v>60</v>
       </c>
@@ -2334,7 +2360,7 @@
         <v>0.87964504737233462</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B25" s="19" t="s">
         <v>61</v>
       </c>
@@ -2380,7 +2406,7 @@
         <v>7203.3637644090004</v>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N26" s="3" t="s">
         <v>42</v>
       </c>
@@ -2403,7 +2429,7 @@
         <v>61.904815039006735</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N27" s="3" t="s">
         <v>38</v>
       </c>
@@ -2426,7 +2452,7 @@
         <v>9.8807884726655857</v>
       </c>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A28" s="4"/>
       <c r="B28" s="4"/>
       <c r="C28" s="9"/>
@@ -2452,7 +2478,7 @@
         <v>4020.725250921625</v>
       </c>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A29" s="4"/>
       <c r="B29" s="4"/>
       <c r="C29" s="9"/>
@@ -2464,7 +2490,7 @@
       <c r="S29" s="3"/>
       <c r="T29" s="3"/>
     </row>
-    <row r="30" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="4"/>
       <c r="B30" s="4"/>
       <c r="C30" s="9"/>
@@ -2478,7 +2504,7 @@
       <c r="S30" s="11"/>
       <c r="T30" s="11"/>
     </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A31" s="5"/>
       <c r="B31" s="5"/>
       <c r="C31" s="6"/>
@@ -2502,7 +2528,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A32" s="7"/>
       <c r="B32" s="7"/>
       <c r="C32" s="7"/>
@@ -2528,7 +2554,7 @@
         <v>1799.9672083200001</v>
       </c>
     </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A33" s="5"/>
       <c r="B33" s="5"/>
       <c r="C33" s="5"/>
@@ -2554,7 +2580,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A34" s="8"/>
       <c r="B34" s="8"/>
       <c r="C34" s="8"/>
@@ -2580,7 +2606,7 @@
         <v>19.661164899999999</v>
       </c>
     </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A35" s="5"/>
       <c r="B35" s="5"/>
       <c r="C35" s="5"/>
@@ -2606,7 +2632,7 @@
         <v>0.207687817</v>
       </c>
     </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A36" s="8"/>
       <c r="B36" s="8"/>
       <c r="C36" s="8"/>
@@ -2632,7 +2658,7 @@
         <v>4.1020808222500005</v>
       </c>
     </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N37" s="3" t="s">
         <v>23</v>
       </c>
@@ -2655,7 +2681,17 @@
         <v>19.453477082999999</v>
       </c>
     </row>
-    <row r="38" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A38" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="B38" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C38" s="36">
+        <f>P20/(P8*3600/1000)</f>
+        <v>0.10637012744588423</v>
+      </c>
       <c r="N38" s="3" t="s">
         <v>24</v>
       </c>
@@ -2678,7 +2714,7 @@
         <v>17.713778155222222</v>
       </c>
     </row>
-    <row r="39" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A39" s="7" t="s">
         <v>44</v>
       </c>
@@ -2711,7 +2747,7 @@
         <v>15.974079227444445</v>
       </c>
     </row>
-    <row r="40" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A40" s="7" t="s">
         <v>45</v>
       </c>
@@ -2719,8 +2755,8 @@
         <v>47</v>
       </c>
       <c r="C40" s="7">
-        <f>P26/1000</f>
-        <v>-2.803449415155216E-2</v>
+        <f>(P16+P17)/(P8*3600/1000)</f>
+        <v>7.833563329433206E-2</v>
       </c>
       <c r="N40" s="3" t="s">
         <v>26</v>
@@ -2744,7 +2780,7 @@
         <v>0.98841122610606125</v>
       </c>
     </row>
-    <row r="41" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A41" s="7" t="s">
         <v>46</v>
       </c>
@@ -2777,7 +2813,7 @@
         <v>3.1058323420000002</v>
       </c>
     </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N42" s="3" t="s">
         <v>28</v>
       </c>
@@ -2800,7 +2836,7 @@
         <v>5.1170056500000003</v>
       </c>
     </row>
-    <row r="43" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N43" s="3" t="s">
         <v>29</v>
       </c>
@@ -2823,7 +2859,7 @@
         <v>14.592057884886959</v>
       </c>
     </row>
-    <row r="44" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N44" s="3" t="s">
         <v>30</v>
       </c>
@@ -2846,7 +2882,7 @@
         <v>3.5572331500000001</v>
       </c>
     </row>
-    <row r="45" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N45" s="3" t="s">
         <v>31</v>
       </c>
@@ -2869,7 +2905,7 @@
         <v>4.2368806800000005</v>
       </c>
     </row>
-    <row r="46" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N46" s="3" t="s">
         <v>32</v>
       </c>
@@ -2892,7 +2928,7 @@
         <v>9.9445346300000001E-2</v>
       </c>
     </row>
-    <row r="47" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N47" s="3" t="s">
         <v>33</v>
       </c>
@@ -2915,7 +2951,7 @@
         <v>38.574472030429632</v>
       </c>
     </row>
-    <row r="48" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N48" s="3" t="s">
         <v>34</v>
       </c>
@@ -2938,7 +2974,7 @@
         <v>0.56964816699999998</v>
       </c>
     </row>
-    <row r="49" spans="14:20" x14ac:dyDescent="0.25">
+    <row r="49" spans="14:20" x14ac:dyDescent="0.3">
       <c r="N49" s="18" t="s">
         <v>58</v>
       </c>
@@ -2961,7 +2997,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="50" spans="14:20" x14ac:dyDescent="0.25">
+    <row r="50" spans="14:20" x14ac:dyDescent="0.3">
       <c r="N50" s="3" t="s">
         <v>35</v>
       </c>
@@ -2984,7 +3020,7 @@
         <v>21030.427199999998</v>
       </c>
     </row>
-    <row r="51" spans="14:20" x14ac:dyDescent="0.25">
+    <row r="51" spans="14:20" x14ac:dyDescent="0.3">
       <c r="N51" s="3" t="s">
         <v>36</v>
       </c>
@@ -3007,7 +3043,7 @@
         <v>-6.4383693151130394</v>
       </c>
     </row>
-    <row r="52" spans="14:20" x14ac:dyDescent="0.25">
+    <row r="52" spans="14:20" x14ac:dyDescent="0.3">
       <c r="N52" s="3"/>
       <c r="O52" s="12"/>
       <c r="P52" s="12"/>
@@ -3024,7 +3060,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="14:20" x14ac:dyDescent="0.25">
+    <row r="53" spans="14:20" x14ac:dyDescent="0.3">
       <c r="N53" s="3" t="s">
         <v>41</v>
       </c>
@@ -3047,7 +3083,7 @@
         <v>0.89878949162663713</v>
       </c>
     </row>
-    <row r="54" spans="14:20" x14ac:dyDescent="0.25">
+    <row r="54" spans="14:20" x14ac:dyDescent="0.3">
       <c r="N54" s="3" t="s">
         <v>37</v>
       </c>
@@ -3070,7 +3106,7 @@
         <v>4336.8956744670004</v>
       </c>
     </row>
-    <row r="55" spans="14:20" x14ac:dyDescent="0.25">
+    <row r="55" spans="14:20" x14ac:dyDescent="0.3">
       <c r="N55" s="3" t="s">
         <v>42</v>
       </c>
@@ -3093,7 +3129,7 @@
         <v>61.926885243577217</v>
       </c>
     </row>
-    <row r="56" spans="14:20" x14ac:dyDescent="0.25">
+    <row r="56" spans="14:20" x14ac:dyDescent="0.3">
       <c r="N56" s="3" t="s">
         <v>38</v>
       </c>
@@ -3116,7 +3152,7 @@
         <v>9.9691968308401844</v>
       </c>
     </row>
-    <row r="57" spans="14:20" x14ac:dyDescent="0.25">
+    <row r="57" spans="14:20" x14ac:dyDescent="0.3">
       <c r="N57" s="3" t="s">
         <v>39</v>
       </c>
@@ -3141,6 +3177,14 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:B5"/>
+    <mergeCell ref="C2:G2"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="F4:F5"/>
+    <mergeCell ref="G4:G5"/>
     <mergeCell ref="A14:G14"/>
     <mergeCell ref="A15:B18"/>
     <mergeCell ref="C15:G15"/>
@@ -3149,14 +3193,6 @@
     <mergeCell ref="E17:E18"/>
     <mergeCell ref="F17:F18"/>
     <mergeCell ref="G17:G18"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:B5"/>
-    <mergeCell ref="C2:G2"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="F4:F5"/>
-    <mergeCell ref="G4:G5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
fixed ranges of oxyfuel by adding extrapolated sizes and costs
</commit_message>
<xml_diff>
--- a/adopt_net0/database/templates/technology_data/Industrial/CementHybridCCS_data/cement_sheet.xlsx
+++ b/adopt_net0/database/templates/technology_data/Industrial/CementHybridCCS_data/cement_sheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\0954659\PycharmProjects\AdOpT-NET0_luca\adopt_net0\database\templates\technology_data\Industrial\CementHybridCCS_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FAE1B19-950B-46D2-A8AD-6DB545E78BF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D196E75-67D7-46C5-8F2F-B7E942B46090}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="4" xr2:uid="{C0ECAA26-0769-408D-9398-31AECF4E3649}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C0ECAA26-0769-408D-9398-31AECF4E3649}"/>
   </bookViews>
   <sheets>
     <sheet name="capex_oxyfuel" sheetId="1" r:id="rId1"/>
@@ -69,6 +69,133 @@
           <t xml:space="preserve">
 In euro totali
 </t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A4" authorId="0" shapeId="0" xr:uid="{1034DA71-6109-44C0-9094-3BCE06243C3C}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Bertoni, L. (Luca):</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+EXTRAPOLATED FOR LARGER SIZES</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Bertoni, L. (Luca)</author>
+  </authors>
+  <commentList>
+    <comment ref="A5" authorId="0" shapeId="0" xr:uid="{59747281-07D3-4DCE-BDD0-69E2E6DC2FBF}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Bertoni, L. (Luca):</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+EXTRAPOLATED FOR LARGER SIZES
+</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Bertoni, L. (Luca)</author>
+  </authors>
+  <commentList>
+    <comment ref="A5" authorId="0" shapeId="0" xr:uid="{85FE4FC7-4322-4255-AC19-69B46725FD92}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Bertoni, L. (Luca):</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+EXTRAPOLATED VALUES</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Bertoni, L. (Luca)</author>
+  </authors>
+  <commentList>
+    <comment ref="A6" authorId="0" shapeId="0" xr:uid="{A4D6E8CB-D7FE-4625-9A12-93585CE13DC0}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Bertoni, L. (Luca):</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+EXTRAPOLATED VALUES</t>
         </r>
       </text>
     </comment>
@@ -620,7 +747,7 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -633,29 +760,23 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="13" xfId="4"/>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="13" xfId="4" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="4" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="2" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="3" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="3" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="4" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="13" xfId="4" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="13" xfId="4" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -692,8 +813,7 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="3" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="13" xfId="4" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Calculation" xfId="5" builtinId="22"/>
@@ -1031,9 +1151,31 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="3">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{13924970-DEDD-4F4D-AF29-711825A865F8}">
+  <we:reference id="WA200009404" version="1.0.0.8" store="Omex" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="WA200009404" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;c842edf6-2ce3-4477-964f-d61e0e183d7e&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D08EB36-8885-41F7-B3E9-60083815A79B}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
@@ -1064,6 +1206,15 @@
         <v>72350000</v>
       </c>
     </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="33">
+        <v>200</v>
+      </c>
+      <c r="B4" s="33">
+        <f>_xlfn.FORECAST.LINEAR($A$4, B2:B3, $A$2:$A$3)</f>
+        <v>104735000</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
@@ -1071,12 +1222,12 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{447E0F8A-1C59-405C-B3D0-EB533A2330E6}">
-  <dimension ref="A1:C4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{447E0F8A-1C59-405C-B3D0-EB533A2330E6}">
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
@@ -1121,15 +1272,25 @@
         <v>26820000.000000007</v>
       </c>
     </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="33">
+        <v>50</v>
+      </c>
+      <c r="B5" s="33">
+        <f>_xlfn.FORECAST.LINEAR($A$5, B3:B4, $A$3:$A$4)</f>
+        <v>30689778.48449932</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E17DFFB0-96B6-4F96-B3DF-E2D36B37C43F}">
-  <dimension ref="A1:D4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E17DFFB0-96B6-4F96-B3DF-E2D36B37C43F}">
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
@@ -1188,19 +1349,37 @@
         <v>71600000</v>
       </c>
     </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="33">
+        <v>200</v>
+      </c>
+      <c r="B5" s="33">
+        <f>_xlfn.FORECAST.LINEAR($A$5, B3:B4, $A$3:$A$4)</f>
+        <v>83350000</v>
+      </c>
+      <c r="C5" s="33">
+        <f t="shared" ref="C5:D5" si="0">_xlfn.FORECAST.LINEAR($A$5, C3:C4, $A$3:$A$4)</f>
+        <v>82950000</v>
+      </c>
+      <c r="D5" s="33">
+        <f t="shared" si="0"/>
+        <v>87500000</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8995DE27-F5E7-40F1-8502-5CC793EB5921}">
-  <dimension ref="A1:D5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8995DE27-F5E7-40F1-8502-5CC793EB5921}">
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1285,8 +1464,26 @@
         <v>19939806.622189701</v>
       </c>
     </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="33">
+        <v>50</v>
+      </c>
+      <c r="B6" s="33">
+        <f>_xlfn.FORECAST.LINEAR($A$6, B4:B5, A4:A5)</f>
+        <v>18648960.688236542</v>
+      </c>
+      <c r="C6" s="33">
+        <f>_xlfn.FORECAST.LINEAR($A$6, C4:C5, A4:A5)</f>
+        <v>21918026.046032257</v>
+      </c>
+      <c r="D6" s="33">
+        <f>_xlfn.FORECAST.LINEAR($A$6, D4:D5, A4:A5)</f>
+        <v>28821920.599393677</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1346,13 +1543,13 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21185F42-04E5-4941-B133-36036095D1EF}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>53</v>
       </c>
@@ -1366,48 +1563,39 @@
         <v>56</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="13" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>52</v>
       </c>
-      <c r="B2" s="14">
+      <c r="B2" s="12">
         <v>0.17050594000000002</v>
       </c>
-      <c r="C2" s="14">
+      <c r="C2" s="12">
         <v>0.120245032</v>
       </c>
-      <c r="D2" s="14">
+      <c r="D2" s="12">
         <v>0.13739152500000001</v>
       </c>
-      <c r="E2" s="13"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="13" t="s">
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>57</v>
       </c>
-      <c r="B3" s="15">
+      <c r="B3" s="13">
         <v>0.11930297990344463</v>
       </c>
-      <c r="C3" s="15">
+      <c r="C3" s="13">
         <v>7.4589551950173874E-2</v>
       </c>
-      <c r="D3" s="15">
+      <c r="D3" s="13">
         <v>8.9737128657946114E-2</v>
       </c>
-      <c r="E3" s="13"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="13"/>
-      <c r="B4" s="13"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="D6" s="35"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="D7" s="35"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D6" s="20"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D7" s="20"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1427,37 +1615,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="16.2" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="25"/>
-      <c r="N1" s="11"/>
-      <c r="O1" s="11" t="s">
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="23"/>
+      <c r="N1" s="10"/>
+      <c r="O1" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="P1" s="11"/>
-      <c r="Q1" s="11"/>
-      <c r="R1" s="11"/>
-      <c r="S1" s="11"/>
+      <c r="P1" s="10"/>
+      <c r="Q1" s="10"/>
+      <c r="R1" s="10"/>
+      <c r="S1" s="10"/>
       <c r="T1" s="3"/>
     </row>
     <row r="2" spans="1:20" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="32" t="s">
+      <c r="B2" s="25"/>
+      <c r="C2" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="33"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="31"/>
       <c r="N2" s="3"/>
       <c r="O2" s="3" t="s">
         <v>17</v>
@@ -1479,8 +1667,8 @@
       </c>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A3" s="28"/>
-      <c r="B3" s="29"/>
+      <c r="A3" s="26"/>
+      <c r="B3" s="27"/>
       <c r="C3" s="1" t="s">
         <v>6</v>
       </c>
@@ -1499,73 +1687,73 @@
       <c r="N3" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="O3" s="12">
+      <c r="O3" s="11">
         <v>3000.0035074612701</v>
       </c>
-      <c r="P3" s="12">
+      <c r="P3" s="11">
         <v>2999.91944736</v>
       </c>
-      <c r="Q3" s="12">
+      <c r="Q3" s="11">
         <v>2999.91944736</v>
       </c>
-      <c r="R3" s="12">
+      <c r="R3" s="11">
         <v>2999.91944736</v>
       </c>
-      <c r="S3" s="12">
+      <c r="S3" s="11">
         <v>2999.91944736</v>
       </c>
-      <c r="T3" s="12">
+      <c r="T3" s="11">
         <v>2999.91944736</v>
       </c>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A4" s="28"/>
-      <c r="B4" s="29"/>
-      <c r="C4" s="34">
+      <c r="A4" s="26"/>
+      <c r="B4" s="27"/>
+      <c r="C4" s="32">
         <v>72.349999999999994</v>
       </c>
-      <c r="D4" s="34">
+      <c r="D4" s="32">
         <v>84.320988516056687</v>
       </c>
-      <c r="E4" s="34">
+      <c r="E4" s="32">
         <v>89.206549352337717</v>
       </c>
-      <c r="F4" s="34">
+      <c r="F4" s="32">
         <v>95.445590190807295</v>
       </c>
-      <c r="G4" s="34">
+      <c r="G4" s="32">
         <v>99.17</v>
       </c>
       <c r="N4" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="O4" s="12">
+      <c r="O4" s="11">
         <v>29.839568333333332</v>
       </c>
-      <c r="P4" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q4" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="R4" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="S4" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="T4" s="12" t="s">
+      <c r="P4" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q4" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="R4" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="S4" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="T4" s="11" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A5" s="30"/>
-      <c r="B5" s="31"/>
-      <c r="C5" s="34"/>
-      <c r="D5" s="34"/>
-      <c r="E5" s="34"/>
-      <c r="F5" s="34"/>
-      <c r="G5" s="34"/>
+      <c r="A5" s="28"/>
+      <c r="B5" s="29"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="32"/>
+      <c r="E5" s="32"/>
+      <c r="F5" s="32"/>
+      <c r="G5" s="32"/>
       <c r="L5">
         <f>1-P6/P5</f>
         <v>0.78184911505744248</v>
@@ -1573,22 +1761,22 @@
       <c r="N5" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="O5" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="P5" s="12">
+      <c r="O5" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="P5" s="11">
         <v>32.665832100000003</v>
       </c>
-      <c r="Q5" s="12">
+      <c r="Q5" s="11">
         <v>32.665832100000003</v>
       </c>
-      <c r="R5" s="12">
+      <c r="R5" s="11">
         <v>32.665832100000003</v>
       </c>
-      <c r="S5" s="12">
+      <c r="S5" s="11">
         <v>32.665832100000003</v>
       </c>
-      <c r="T5" s="12">
+      <c r="T5" s="11">
         <v>32.665832100000003</v>
       </c>
     </row>
@@ -1611,29 +1799,29 @@
         <f t="shared" si="0"/>
         <v>19.535058601920007</v>
       </c>
-      <c r="G6" s="21">
+      <c r="G6" s="18">
         <f t="shared" si="0"/>
         <v>24.418823252400006</v>
       </c>
       <c r="N6" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="O6" s="12">
+      <c r="O6" s="11">
         <v>29.839568333333332</v>
       </c>
-      <c r="P6" s="12">
+      <c r="P6" s="11">
         <v>7.1260801800000015</v>
       </c>
-      <c r="Q6" s="12">
+      <c r="Q6" s="11">
         <v>5.0911782423000007</v>
       </c>
-      <c r="R6" s="12">
+      <c r="R6" s="11">
         <v>3.7345769505000006</v>
       </c>
-      <c r="S6" s="12">
+      <c r="S6" s="11">
         <v>1.6996750128</v>
       </c>
-      <c r="T6" s="12">
+      <c r="T6" s="11">
         <v>0.343073721</v>
       </c>
     </row>
@@ -1661,22 +1849,22 @@
       <c r="N7" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="O7" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="P7" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q7" s="12">
+      <c r="O7" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="P7" s="11">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="11">
         <v>2.0349019377000008</v>
       </c>
-      <c r="R7" s="12">
+      <c r="R7" s="11">
         <v>3.3915032295000009</v>
       </c>
-      <c r="S7" s="12">
+      <c r="S7" s="11">
         <v>5.4264051672000013</v>
       </c>
-      <c r="T7" s="12">
+      <c r="T7" s="11">
         <v>6.7830064590000019</v>
       </c>
     </row>
@@ -1704,22 +1892,22 @@
       <c r="N8" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="O8" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="P8" s="12">
+      <c r="O8" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="P8" s="11">
         <v>25.53975192</v>
       </c>
-      <c r="Q8" s="12">
+      <c r="Q8" s="11">
         <v>27.574653857700003</v>
       </c>
-      <c r="R8" s="12">
+      <c r="R8" s="11">
         <v>28.931255149500004</v>
       </c>
-      <c r="S8" s="12">
+      <c r="S8" s="11">
         <v>30.966157087200003</v>
       </c>
-      <c r="T8" s="12">
+      <c r="T8" s="11">
         <v>32.322758379</v>
       </c>
     </row>
@@ -1746,27 +1934,27 @@
       <c r="N9" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="O9" s="12">
-        <v>0</v>
-      </c>
-      <c r="P9" s="12">
+      <c r="O9" s="11">
+        <v>0</v>
+      </c>
+      <c r="P9" s="11">
         <v>22.71348815333333</v>
       </c>
-      <c r="Q9" s="12">
+      <c r="Q9" s="11">
         <v>24.748390091033333</v>
       </c>
-      <c r="R9" s="12">
+      <c r="R9" s="11">
         <v>26.104991382833333</v>
       </c>
-      <c r="S9" s="12">
+      <c r="S9" s="11">
         <v>28.139893320533332</v>
       </c>
-      <c r="T9" s="12">
+      <c r="T9" s="11">
         <v>29.496494612333333</v>
       </c>
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="16" t="s">
         <v>59</v>
       </c>
       <c r="C10">
@@ -1791,27 +1979,27 @@
       <c r="N10" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="O10" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="P10" s="12">
+      <c r="O10" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="P10" s="11">
         <v>19.887224386666659</v>
       </c>
-      <c r="Q10" s="12">
+      <c r="Q10" s="11">
         <v>21.922126324366658</v>
       </c>
-      <c r="R10" s="12">
+      <c r="R10" s="11">
         <v>23.278727616166663</v>
       </c>
-      <c r="S10" s="12">
+      <c r="S10" s="11">
         <v>25.313629553866662</v>
       </c>
-      <c r="T10" s="12">
+      <c r="T10" s="11">
         <v>26.670230845666659</v>
       </c>
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="16" t="s">
         <v>60</v>
       </c>
       <c r="C11">
@@ -1837,68 +2025,68 @@
       <c r="N11" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="O11" s="12">
-        <v>0</v>
-      </c>
-      <c r="P11" s="12">
+      <c r="O11" s="11">
+        <v>0</v>
+      </c>
+      <c r="P11" s="11">
         <v>0.76118688781299948</v>
       </c>
-      <c r="Q11" s="12">
+      <c r="Q11" s="11">
         <v>0.82938163898930395</v>
       </c>
-      <c r="R11" s="12">
+      <c r="R11" s="11">
         <v>0.87484480644017359</v>
       </c>
-      <c r="S11" s="12">
+      <c r="S11" s="11">
         <v>0.94303955761647806</v>
       </c>
-      <c r="T11" s="12">
+      <c r="T11" s="11">
         <v>0.98850272506734771</v>
       </c>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="C12" s="20">
+      <c r="C12" s="17">
         <f>C10/C4</f>
         <v>0.16447823082239116</v>
       </c>
-      <c r="D12" s="17">
+      <c r="D12" s="14">
         <f>D11*10^6/D7</f>
         <v>1.8377763850070759E-2</v>
       </c>
-      <c r="E12" s="17">
+      <c r="E12" s="14">
         <f t="shared" ref="E12:G12" si="4">E11*10^6/E7</f>
         <v>1.8983719224576746E-2</v>
       </c>
-      <c r="F12" s="17">
+      <c r="F12" s="14">
         <f t="shared" si="4"/>
         <v>2.1649154486600396E-2</v>
       </c>
-      <c r="G12" s="17">
+      <c r="G12" s="14">
         <f t="shared" si="4"/>
         <v>2.2744220730797883E-2</v>
       </c>
       <c r="N12" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="O12" s="12">
+      <c r="O12" s="11">
         <v>4.0947408000000003</v>
       </c>
-      <c r="P12" s="12">
+      <c r="P12" s="11">
         <v>5.1419803699999997</v>
       </c>
-      <c r="Q12" s="12">
+      <c r="Q12" s="11">
         <v>5.1419803699999997</v>
       </c>
-      <c r="R12" s="12">
+      <c r="R12" s="11">
         <v>5.1419803699999997</v>
       </c>
-      <c r="S12" s="12">
+      <c r="S12" s="11">
         <v>5.1419803699999997</v>
       </c>
-      <c r="T12" s="12">
+      <c r="T12" s="11">
         <v>5.1419803699999997</v>
       </c>
     </row>
@@ -1906,94 +2094,94 @@
       <c r="N13" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O13" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="P13" s="12">
+      <c r="O13" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="P13" s="11">
         <v>8.4990979400000004</v>
       </c>
-      <c r="Q13" s="12">
+      <c r="Q13" s="11">
         <v>8.4990979400000004</v>
       </c>
-      <c r="R13" s="12">
+      <c r="R13" s="11">
         <v>8.4990979400000004</v>
       </c>
-      <c r="S13" s="12">
+      <c r="S13" s="11">
         <v>8.4990979400000004</v>
       </c>
-      <c r="T13" s="12">
+      <c r="T13" s="11">
         <v>8.4990979400000004</v>
       </c>
     </row>
     <row r="14" spans="1:20" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A14" s="23" t="s">
+      <c r="A14" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="24"/>
-      <c r="C14" s="24"/>
-      <c r="D14" s="24"/>
-      <c r="E14" s="24"/>
-      <c r="F14" s="24"/>
-      <c r="G14" s="25"/>
+      <c r="B14" s="22"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="22"/>
+      <c r="G14" s="23"/>
       <c r="N14" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="O14" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="P14" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q14" s="12">
+      <c r="O14" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="P14" s="11">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="11">
         <v>7.2054566119658183</v>
       </c>
-      <c r="R14" s="12">
+      <c r="R14" s="11">
         <v>12.009094353276362</v>
       </c>
-      <c r="S14" s="12">
+      <c r="S14" s="11">
         <v>19.214550965242179</v>
       </c>
-      <c r="T14" s="12">
+      <c r="T14" s="11">
         <v>24.018188706552724</v>
       </c>
     </row>
     <row r="15" spans="1:20" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A15" s="26" t="s">
+      <c r="A15" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="B15" s="27"/>
-      <c r="C15" s="32" t="s">
+      <c r="B15" s="25"/>
+      <c r="C15" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="D15" s="32"/>
-      <c r="E15" s="32"/>
-      <c r="F15" s="32"/>
-      <c r="G15" s="33"/>
+      <c r="D15" s="30"/>
+      <c r="E15" s="30"/>
+      <c r="F15" s="30"/>
+      <c r="G15" s="31"/>
       <c r="N15" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="O15" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="P15" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q15" s="12">
+      <c r="O15" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="P15" s="11">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="11">
         <v>3.5409355499999999</v>
       </c>
-      <c r="R15" s="12">
+      <c r="R15" s="11">
         <v>3.5409355499999999</v>
       </c>
-      <c r="S15" s="12">
+      <c r="S15" s="11">
         <v>3.5409355499999999</v>
       </c>
-      <c r="T15" s="12">
+      <c r="T15" s="11">
         <v>3.5409355499999999</v>
       </c>
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A16" s="28"/>
-      <c r="B16" s="29"/>
+      <c r="A16" s="26"/>
+      <c r="B16" s="27"/>
       <c r="C16" s="1" t="s">
         <v>6</v>
       </c>
@@ -2012,104 +2200,104 @@
       <c r="N16" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="O16" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="P16" s="12">
+      <c r="O16" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="P16" s="11">
         <v>7.0372530900000001</v>
       </c>
-      <c r="Q16" s="12">
+      <c r="Q16" s="11">
         <v>7.0372530900000001</v>
       </c>
-      <c r="R16" s="12">
+      <c r="R16" s="11">
         <v>7.0372530900000001</v>
       </c>
-      <c r="S16" s="12">
+      <c r="S16" s="11">
         <v>7.0372530900000001</v>
       </c>
-      <c r="T16" s="12">
+      <c r="T16" s="11">
         <v>7.0372530900000001</v>
       </c>
     </row>
     <row r="17" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A17" s="28"/>
-      <c r="B17" s="29"/>
-      <c r="C17" s="34">
+      <c r="A17" s="26"/>
+      <c r="B17" s="27"/>
+      <c r="C17" s="32">
         <v>50.76</v>
       </c>
-      <c r="D17" s="34">
+      <c r="D17" s="32">
         <v>64.722331812465825</v>
       </c>
-      <c r="E17" s="34">
+      <c r="E17" s="32">
         <v>68.47234583745032</v>
       </c>
-      <c r="F17" s="34">
+      <c r="F17" s="32">
         <v>73.261251641870047</v>
       </c>
-      <c r="G17" s="34">
+      <c r="G17" s="32">
         <v>76.12</v>
       </c>
       <c r="N17" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="O17" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="P17" s="12">
+      <c r="O17" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="P17" s="11">
         <v>0.16516841700000001</v>
       </c>
-      <c r="Q17" s="12">
+      <c r="Q17" s="11">
         <v>0.16516841700000001</v>
       </c>
-      <c r="R17" s="12">
+      <c r="R17" s="11">
         <v>0.16516841700000001</v>
       </c>
-      <c r="S17" s="12">
+      <c r="S17" s="11">
         <v>0.16516841700000001</v>
       </c>
-      <c r="T17" s="12">
+      <c r="T17" s="11">
         <v>0.16516841700000001</v>
       </c>
     </row>
     <row r="18" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A18" s="30"/>
-      <c r="B18" s="31"/>
-      <c r="C18" s="34"/>
-      <c r="D18" s="34"/>
-      <c r="E18" s="34"/>
-      <c r="F18" s="34"/>
-      <c r="G18" s="34"/>
+      <c r="A18" s="28"/>
+      <c r="B18" s="29"/>
+      <c r="C18" s="32"/>
+      <c r="D18" s="32"/>
+      <c r="E18" s="32"/>
+      <c r="F18" s="32"/>
+      <c r="G18" s="32"/>
       <c r="N18" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="O18" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="P18" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q18" s="12">
+      <c r="O18" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="P18" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q18" s="11">
         <v>38.587338925408297</v>
       </c>
-      <c r="R18" s="12">
+      <c r="R18" s="11">
         <v>38.587338925408297</v>
       </c>
-      <c r="S18" s="12">
+      <c r="S18" s="11">
         <v>38.587338925408297</v>
       </c>
-      <c r="T18" s="12">
+      <c r="T18" s="11">
         <v>38.587338925408297</v>
       </c>
     </row>
     <row r="19" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A19" s="10"/>
+      <c r="A19" s="3"/>
       <c r="B19" s="7" t="s">
         <v>13</v>
       </c>
       <c r="C19" s="7">
         <v>0</v>
       </c>
-      <c r="D19" s="21">
+      <c r="D19" s="18">
         <f>Q36*3600/1000</f>
         <v>4.4302472880300003</v>
       </c>
@@ -2117,33 +2305,33 @@
         <f t="shared" ref="E19:G19" si="5">R36*3600/1000</f>
         <v>7.3837454800500009</v>
       </c>
-      <c r="F19" s="22">
+      <c r="F19" s="19">
         <f>S36*3600/1000</f>
         <v>11.81399276808</v>
       </c>
-      <c r="G19" s="21">
+      <c r="G19" s="18">
         <f t="shared" si="5"/>
         <v>14.767490960100002</v>
       </c>
       <c r="N19" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="O19" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="P19" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q19" s="12">
+      <c r="O19" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="P19" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q19" s="11">
         <v>0.28267722270000001</v>
       </c>
-      <c r="R19" s="12">
+      <c r="R19" s="11">
         <v>0.47112870450000005</v>
       </c>
-      <c r="S19" s="12">
+      <c r="S19" s="11">
         <v>0.75380592720000006</v>
       </c>
-      <c r="T19" s="12">
+      <c r="T19" s="11">
         <v>0.9422574090000001</v>
       </c>
     </row>
@@ -2168,25 +2356,25 @@
         <f t="shared" si="6"/>
         <v>25360000.000000007</v>
       </c>
-      <c r="N20" s="18" t="s">
+      <c r="N20" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="O20" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="P20" s="16">
+      <c r="O20" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="P20" s="11">
         <v>9.7799999999999994</v>
       </c>
-      <c r="Q20" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="R20" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="S20" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="T20" s="16" t="s">
+      <c r="Q20" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="R20" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="S20" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="T20" s="11" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2214,22 +2402,22 @@
       <c r="N21" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="O21" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="P21" s="12">
+      <c r="O21" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="P21" s="11">
         <v>34915.217199999999</v>
       </c>
-      <c r="Q21" s="12">
+      <c r="Q21" s="11">
         <v>34915.217199999999</v>
       </c>
-      <c r="R21" s="12">
+      <c r="R21" s="11">
         <v>34915.217199999999</v>
       </c>
-      <c r="S21" s="12">
+      <c r="S21" s="11">
         <v>34915.217199999999</v>
       </c>
-      <c r="T21" s="12">
+      <c r="T21" s="11">
         <v>34915.217199999999</v>
       </c>
     </row>
@@ -2256,27 +2444,27 @@
       <c r="N22" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="O22" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="P22" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q22" s="12">
+      <c r="O22" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="P22" s="11">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="11">
         <v>-27.709760588034182</v>
       </c>
-      <c r="R22" s="12">
+      <c r="R22" s="11">
         <v>-22.90612284672364</v>
       </c>
-      <c r="S22" s="12">
+      <c r="S22" s="11">
         <v>-15.700666234757822</v>
       </c>
-      <c r="T22" s="12">
+      <c r="T22" s="11">
         <v>-10.897028493447277</v>
       </c>
     </row>
     <row r="23" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="B23" s="19" t="s">
+      <c r="B23" s="16" t="s">
         <v>59</v>
       </c>
       <c r="C23">
@@ -2294,28 +2482,28 @@
       <c r="G23">
         <v>9.98</v>
       </c>
-      <c r="N23" s="18" t="s">
+      <c r="N23" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="O23" s="16"/>
-      <c r="P23" s="16">
+      <c r="O23" s="11"/>
+      <c r="P23" s="11">
         <v>9.7799999999999994</v>
       </c>
-      <c r="Q23" s="16">
-        <v>0</v>
-      </c>
-      <c r="R23" s="16">
-        <v>0</v>
-      </c>
-      <c r="S23" s="16">
-        <v>0</v>
-      </c>
-      <c r="T23" s="16">
+      <c r="Q23" s="11">
+        <v>0</v>
+      </c>
+      <c r="R23" s="11">
+        <v>0</v>
+      </c>
+      <c r="S23" s="11">
+        <v>0</v>
+      </c>
+      <c r="T23" s="11">
         <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="B24" s="19" t="s">
+      <c r="B24" s="16" t="s">
         <v>60</v>
       </c>
       <c r="C24">
@@ -2341,68 +2529,68 @@
       <c r="N24" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="O24" s="12">
-        <v>0</v>
-      </c>
-      <c r="P24" s="12">
+      <c r="O24" s="11">
+        <v>0</v>
+      </c>
+      <c r="P24" s="11">
         <v>1.1132666603247092</v>
       </c>
-      <c r="Q24" s="12">
+      <c r="Q24" s="11">
         <v>1.0311119215576452</v>
       </c>
-      <c r="R24" s="12">
+      <c r="R24" s="11">
         <v>0.98276255829817882</v>
       </c>
-      <c r="S24" s="12">
+      <c r="S24" s="11">
         <v>0.9181815568988605</v>
       </c>
-      <c r="T24" s="12">
+      <c r="T24" s="11">
         <v>0.87964504737233462</v>
       </c>
     </row>
     <row r="25" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="B25" s="19" t="s">
+      <c r="B25" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="C25" s="20">
+      <c r="C25" s="17">
         <f>C10/C4</f>
         <v>0.16447823082239116</v>
       </c>
-      <c r="D25" s="17">
+      <c r="D25" s="14">
         <f>D24*10^6/D20</f>
         <v>2.578365883545217E-2</v>
       </c>
-      <c r="E25" s="17">
+      <c r="E25" s="14">
         <f t="shared" ref="E25" si="11">E24*10^6/E20</f>
         <v>2.4841430041958639E-2</v>
       </c>
-      <c r="F25" s="17">
+      <c r="F25" s="14">
         <f t="shared" ref="F25" si="12">F24*10^6/F20</f>
         <v>2.5776343877722045E-2</v>
       </c>
-      <c r="G25" s="17">
+      <c r="G25" s="14">
         <f t="shared" ref="G25" si="13">G24*10^6/G20</f>
         <v>2.641955835962144E-2</v>
       </c>
       <c r="N25" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="O25" s="12">
-        <v>0</v>
-      </c>
-      <c r="P25" s="12">
+      <c r="O25" s="11">
+        <v>0</v>
+      </c>
+      <c r="P25" s="11">
         <v>-2577.5784929999991</v>
       </c>
-      <c r="Q25" s="12">
+      <c r="Q25" s="11">
         <v>7202.7041842227</v>
       </c>
-      <c r="R25" s="12">
+      <c r="R25" s="11">
         <v>7202.8926357045002</v>
       </c>
-      <c r="S25" s="12">
+      <c r="S25" s="11">
         <v>7203.1753129272001</v>
       </c>
-      <c r="T25" s="12">
+      <c r="T25" s="11">
         <v>7203.3637644090004</v>
       </c>
     </row>
@@ -2410,22 +2598,22 @@
       <c r="N26" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="O26" s="12">
-        <v>0</v>
-      </c>
-      <c r="P26" s="12">
+      <c r="O26" s="11">
+        <v>0</v>
+      </c>
+      <c r="P26" s="11">
         <v>-28.03449415155216</v>
       </c>
-      <c r="Q26" s="12">
+      <c r="Q26" s="11">
         <v>72.557616592724315</v>
       </c>
-      <c r="R26" s="12">
+      <c r="R26" s="11">
         <v>69.157162369172056</v>
       </c>
-      <c r="S26" s="12">
+      <c r="S26" s="11">
         <v>64.615122429761868</v>
       </c>
-      <c r="T26" s="12">
+      <c r="T26" s="11">
         <v>61.904815039006735</v>
       </c>
     </row>
@@ -2433,22 +2621,22 @@
       <c r="N27" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="O27" s="12">
+      <c r="O27" s="11">
         <v>859.37856325432426</v>
       </c>
-      <c r="P27" s="12">
+      <c r="P27" s="11">
         <v>205.23661996785438</v>
       </c>
-      <c r="Q27" s="12">
+      <c r="Q27" s="11">
         <v>146.62987051929775</v>
       </c>
-      <c r="R27" s="12">
+      <c r="R27" s="11">
         <v>107.55870422026</v>
       </c>
-      <c r="S27" s="12">
+      <c r="S27" s="11">
         <v>48.951954771703335</v>
       </c>
-      <c r="T27" s="12">
+      <c r="T27" s="11">
         <v>9.8807884726655857</v>
       </c>
     </row>
@@ -2459,22 +2647,22 @@
       <c r="N28" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="O28" s="12">
+      <c r="O28" s="11">
         <v>3201.7559829909646</v>
       </c>
-      <c r="P28" s="12">
+      <c r="P28" s="11">
         <v>4020.725250921625</v>
       </c>
-      <c r="Q28" s="12">
+      <c r="Q28" s="11">
         <v>4020.725250921625</v>
       </c>
-      <c r="R28" s="12">
+      <c r="R28" s="11">
         <v>4020.725250921625</v>
       </c>
-      <c r="S28" s="12">
+      <c r="S28" s="11">
         <v>4020.725250921625</v>
       </c>
-      <c r="T28" s="12">
+      <c r="T28" s="11">
         <v>4020.725250921625</v>
       </c>
     </row>
@@ -2494,15 +2682,15 @@
       <c r="A30" s="4"/>
       <c r="B30" s="4"/>
       <c r="C30" s="9"/>
-      <c r="N30" s="11"/>
-      <c r="O30" s="11" t="s">
+      <c r="N30" s="10"/>
+      <c r="O30" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="P30" s="11"/>
-      <c r="Q30" s="11"/>
-      <c r="R30" s="11"/>
-      <c r="S30" s="11"/>
-      <c r="T30" s="11"/>
+      <c r="P30" s="10"/>
+      <c r="Q30" s="10"/>
+      <c r="R30" s="10"/>
+      <c r="S30" s="10"/>
+      <c r="T30" s="10"/>
     </row>
     <row r="31" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A31" s="5"/>
@@ -2535,22 +2723,22 @@
       <c r="N32" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="O32" s="12">
+      <c r="O32" s="11">
         <v>1800.17599</v>
       </c>
-      <c r="P32" s="12">
+      <c r="P32" s="11">
         <v>1799.9672083200001</v>
       </c>
-      <c r="Q32" s="12">
+      <c r="Q32" s="11">
         <v>1799.9672083200001</v>
       </c>
-      <c r="R32" s="12">
+      <c r="R32" s="11">
         <v>1799.9672083200001</v>
       </c>
-      <c r="S32" s="12">
+      <c r="S32" s="11">
         <v>1799.9672083200001</v>
       </c>
-      <c r="T32" s="12">
+      <c r="T32" s="11">
         <v>1799.9672083200001</v>
       </c>
     </row>
@@ -2561,22 +2749,22 @@
       <c r="N33" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="O33" s="12">
+      <c r="O33" s="11">
         <v>17.921465972222222</v>
       </c>
-      <c r="P33" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q33" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="R33" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="S33" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="T33" s="12" t="s">
+      <c r="P33" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q33" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="R33" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="S33" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="T33" s="11" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2587,22 +2775,22 @@
       <c r="N34" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="O34" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="P34" s="12">
+      <c r="O34" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="P34" s="11">
         <v>19.661164899999999</v>
       </c>
-      <c r="Q34" s="12">
+      <c r="Q34" s="11">
         <v>19.661164899999999</v>
       </c>
-      <c r="R34" s="12">
+      <c r="R34" s="11">
         <v>19.661164899999999</v>
       </c>
-      <c r="S34" s="12">
+      <c r="S34" s="11">
         <v>19.661164899999999</v>
       </c>
-      <c r="T34" s="12">
+      <c r="T34" s="11">
         <v>19.661164899999999</v>
       </c>
     </row>
@@ -2613,22 +2801,22 @@
       <c r="N35" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="O35" s="12">
+      <c r="O35" s="11">
         <v>17.921465972222222</v>
       </c>
-      <c r="P35" s="12">
+      <c r="P35" s="11">
         <v>4.3097686392500005</v>
       </c>
-      <c r="Q35" s="12">
+      <c r="Q35" s="11">
         <v>3.0791443925750004</v>
       </c>
-      <c r="R35" s="12">
+      <c r="R35" s="11">
         <v>2.2587282281250003</v>
       </c>
-      <c r="S35" s="12">
+      <c r="S35" s="11">
         <v>1.0281039814499999</v>
       </c>
-      <c r="T35" s="12">
+      <c r="T35" s="11">
         <v>0.207687817</v>
       </c>
     </row>
@@ -2639,22 +2827,22 @@
       <c r="N36" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="O36" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="P36" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q36" s="12">
+      <c r="O36" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="P36" s="11">
+        <v>0</v>
+      </c>
+      <c r="Q36" s="11">
         <v>1.2306242466750001</v>
       </c>
-      <c r="R36" s="12">
+      <c r="R36" s="11">
         <v>2.0510404111250002</v>
       </c>
-      <c r="S36" s="12">
+      <c r="S36" s="11">
         <v>3.2816646578000004</v>
       </c>
-      <c r="T36" s="12">
+      <c r="T36" s="11">
         <v>4.1020808222500005</v>
       </c>
     </row>
@@ -2662,22 +2850,22 @@
       <c r="N37" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="O37" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="P37" s="12">
+      <c r="O37" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="P37" s="11">
         <v>15.351396260749999</v>
       </c>
-      <c r="Q37" s="12">
+      <c r="Q37" s="11">
         <v>16.582020507425</v>
       </c>
-      <c r="R37" s="12">
+      <c r="R37" s="11">
         <v>17.402436671874998</v>
       </c>
-      <c r="S37" s="12">
+      <c r="S37" s="11">
         <v>18.633060918550001</v>
       </c>
-      <c r="T37" s="12">
+      <c r="T37" s="11">
         <v>19.453477082999999</v>
       </c>
     </row>
@@ -2688,29 +2876,29 @@
       <c r="B38" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="C38" s="36">
+      <c r="C38" s="7">
         <f>P20/(P8*3600/1000)</f>
         <v>0.10637012744588423</v>
       </c>
       <c r="N38" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="O38" s="12">
-        <v>0</v>
-      </c>
-      <c r="P38" s="12">
+      <c r="O38" s="11">
+        <v>0</v>
+      </c>
+      <c r="P38" s="11">
         <v>13.611697332972222</v>
       </c>
-      <c r="Q38" s="12">
+      <c r="Q38" s="11">
         <v>14.842321579647223</v>
       </c>
-      <c r="R38" s="12">
+      <c r="R38" s="11">
         <v>15.662737744097221</v>
       </c>
-      <c r="S38" s="12">
+      <c r="S38" s="11">
         <v>16.893361990772224</v>
       </c>
-      <c r="T38" s="12">
+      <c r="T38" s="11">
         <v>17.713778155222222</v>
       </c>
     </row>
@@ -2728,22 +2916,22 @@
       <c r="N39" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="O39" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="P39" s="12">
+      <c r="O39" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="P39" s="11">
         <v>11.871998405194446</v>
       </c>
-      <c r="Q39" s="12">
+      <c r="Q39" s="11">
         <v>13.102622651869446</v>
       </c>
-      <c r="R39" s="12">
+      <c r="R39" s="11">
         <v>13.923038816319444</v>
       </c>
-      <c r="S39" s="12">
+      <c r="S39" s="11">
         <v>15.153663062994447</v>
       </c>
-      <c r="T39" s="12">
+      <c r="T39" s="11">
         <v>15.974079227444445</v>
       </c>
     </row>
@@ -2761,22 +2949,22 @@
       <c r="N40" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="O40" s="12">
-        <v>0</v>
-      </c>
-      <c r="P40" s="12">
+      <c r="O40" s="11">
+        <v>0</v>
+      </c>
+      <c r="P40" s="11">
         <v>0.75951919078885499</v>
       </c>
-      <c r="Q40" s="12">
+      <c r="Q40" s="11">
         <v>0.8281868013840169</v>
       </c>
-      <c r="R40" s="12">
+      <c r="R40" s="11">
         <v>0.87396520844745806</v>
       </c>
-      <c r="S40" s="12">
+      <c r="S40" s="11">
         <v>0.94263281904262008</v>
       </c>
-      <c r="T40" s="12">
+      <c r="T40" s="11">
         <v>0.98841122610606125</v>
       </c>
     </row>
@@ -2794,22 +2982,22 @@
       <c r="N41" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="O41" s="12">
+      <c r="O41" s="11">
         <v>2.4618330500000001</v>
       </c>
-      <c r="P41" s="12">
+      <c r="P41" s="11">
         <v>3.1058323420000002</v>
       </c>
-      <c r="Q41" s="12">
+      <c r="Q41" s="11">
         <v>3.1058323420000002</v>
       </c>
-      <c r="R41" s="12">
+      <c r="R41" s="11">
         <v>3.1058323420000002</v>
       </c>
-      <c r="S41" s="12">
+      <c r="S41" s="11">
         <v>3.1058323420000002</v>
       </c>
-      <c r="T41" s="12">
+      <c r="T41" s="11">
         <v>3.1058323420000002</v>
       </c>
     </row>
@@ -2817,22 +3005,22 @@
       <c r="N42" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O42" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="P42" s="12">
+      <c r="O42" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="P42" s="11">
         <v>5.1170056500000003</v>
       </c>
-      <c r="Q42" s="12">
+      <c r="Q42" s="11">
         <v>5.1170056500000003</v>
       </c>
-      <c r="R42" s="12">
+      <c r="R42" s="11">
         <v>5.1170056500000003</v>
       </c>
-      <c r="S42" s="12">
+      <c r="S42" s="11">
         <v>5.1170056500000003</v>
       </c>
-      <c r="T42" s="12">
+      <c r="T42" s="11">
         <v>5.1170056500000003</v>
       </c>
     </row>
@@ -2840,22 +3028,22 @@
       <c r="N43" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="O43" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="P43" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q43" s="12">
+      <c r="O43" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="P43" s="11">
+        <v>0</v>
+      </c>
+      <c r="Q43" s="11">
         <v>4.3776173654660875</v>
       </c>
-      <c r="R43" s="12">
+      <c r="R43" s="11">
         <v>7.2960289424434794</v>
       </c>
-      <c r="S43" s="12">
+      <c r="S43" s="11">
         <v>11.673646307909568</v>
       </c>
-      <c r="T43" s="12">
+      <c r="T43" s="11">
         <v>14.592057884886959</v>
       </c>
     </row>
@@ -2863,22 +3051,22 @@
       <c r="N44" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="O44" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="P44" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q44" s="12">
+      <c r="O44" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="P44" s="11">
+        <v>0</v>
+      </c>
+      <c r="Q44" s="11">
         <v>3.5572331500000001</v>
       </c>
-      <c r="R44" s="12">
+      <c r="R44" s="11">
         <v>3.5572331500000001</v>
       </c>
-      <c r="S44" s="12">
+      <c r="S44" s="11">
         <v>3.5572331500000001</v>
       </c>
-      <c r="T44" s="12">
+      <c r="T44" s="11">
         <v>3.5572331500000001</v>
       </c>
     </row>
@@ -2886,22 +3074,22 @@
       <c r="N45" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="O45" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="P45" s="12">
+      <c r="O45" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="P45" s="11">
         <v>4.2368806800000005</v>
       </c>
-      <c r="Q45" s="12">
+      <c r="Q45" s="11">
         <v>4.2368806800000005</v>
       </c>
-      <c r="R45" s="12">
+      <c r="R45" s="11">
         <v>4.2368806800000005</v>
       </c>
-      <c r="S45" s="12">
+      <c r="S45" s="11">
         <v>4.2368806800000005</v>
       </c>
-      <c r="T45" s="12">
+      <c r="T45" s="11">
         <v>4.2368806800000005</v>
       </c>
     </row>
@@ -2909,22 +3097,22 @@
       <c r="N46" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="O46" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="P46" s="12">
+      <c r="O46" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="P46" s="11">
         <v>9.9445346300000001E-2</v>
       </c>
-      <c r="Q46" s="12">
+      <c r="Q46" s="11">
         <v>9.9445346300000001E-2</v>
       </c>
-      <c r="R46" s="12">
+      <c r="R46" s="11">
         <v>9.9445346300000001E-2</v>
       </c>
-      <c r="S46" s="12">
+      <c r="S46" s="11">
         <v>9.9445346300000001E-2</v>
       </c>
-      <c r="T46" s="12">
+      <c r="T46" s="11">
         <v>9.9445346300000001E-2</v>
       </c>
     </row>
@@ -2932,22 +3120,22 @@
       <c r="N47" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="O47" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="P47" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q47" s="12">
+      <c r="O47" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="P47" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q47" s="11">
         <v>38.574472030429632</v>
       </c>
-      <c r="R47" s="12">
+      <c r="R47" s="11">
         <v>38.574472030429632</v>
       </c>
-      <c r="S47" s="12">
+      <c r="S47" s="11">
         <v>38.574472030429632</v>
       </c>
-      <c r="T47" s="12">
+      <c r="T47" s="11">
         <v>38.574472030429632</v>
       </c>
     </row>
@@ -2955,45 +3143,45 @@
       <c r="N48" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="O48" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="P48" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q48" s="12">
+      <c r="O48" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="P48" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q48" s="11">
         <v>0.17089445010000001</v>
       </c>
-      <c r="R48" s="12">
+      <c r="R48" s="11">
         <v>0.28482408349999999</v>
       </c>
-      <c r="S48" s="12">
+      <c r="S48" s="11">
         <v>0.45571853359999992</v>
       </c>
-      <c r="T48" s="12">
+      <c r="T48" s="11">
         <v>0.56964816699999998</v>
       </c>
     </row>
     <row r="49" spans="14:20" x14ac:dyDescent="0.3">
-      <c r="N49" s="18" t="s">
+      <c r="N49" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="O49" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="P49" s="16">
+      <c r="O49" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="P49" s="11">
         <v>5.89</v>
       </c>
-      <c r="Q49" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="R49" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="S49" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="T49" s="16" t="s">
+      <c r="Q49" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="R49" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="S49" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="T49" s="11" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3001,22 +3189,22 @@
       <c r="N50" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="O50" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="P50" s="12">
+      <c r="O50" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="P50" s="11">
         <v>21030.427199999998</v>
       </c>
-      <c r="Q50" s="12">
+      <c r="Q50" s="11">
         <v>21030.427199999998</v>
       </c>
-      <c r="R50" s="12">
+      <c r="R50" s="11">
         <v>21030.427199999998</v>
       </c>
-      <c r="S50" s="12">
+      <c r="S50" s="11">
         <v>21030.427199999998</v>
       </c>
-      <c r="T50" s="12">
+      <c r="T50" s="11">
         <v>21030.427199999998</v>
       </c>
     </row>
@@ -3024,39 +3212,39 @@
       <c r="N51" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="O51" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="P51" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q51" s="12">
+      <c r="O51" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="P51" s="11">
+        <v>0</v>
+      </c>
+      <c r="Q51" s="11">
         <v>-16.652809834533912</v>
       </c>
-      <c r="R51" s="12">
+      <c r="R51" s="11">
         <v>-13.734398257556519</v>
       </c>
-      <c r="S51" s="12">
+      <c r="S51" s="11">
         <v>-9.3567808920904305</v>
       </c>
-      <c r="T51" s="12">
+      <c r="T51" s="11">
         <v>-6.4383693151130394</v>
       </c>
     </row>
     <row r="52" spans="14:20" x14ac:dyDescent="0.3">
       <c r="N52" s="3"/>
-      <c r="O52" s="12"/>
-      <c r="P52" s="12"/>
-      <c r="Q52" s="12">
-        <v>0</v>
-      </c>
-      <c r="R52" s="12">
-        <v>0</v>
-      </c>
-      <c r="S52" s="12">
-        <v>0</v>
-      </c>
-      <c r="T52" s="12">
+      <c r="O52" s="11"/>
+      <c r="P52" s="11"/>
+      <c r="Q52" s="11">
+        <v>0</v>
+      </c>
+      <c r="R52" s="11">
+        <v>0</v>
+      </c>
+      <c r="S52" s="11">
+        <v>0</v>
+      </c>
+      <c r="T52" s="11">
         <v>0</v>
       </c>
     </row>
@@ -3064,22 +3252,22 @@
       <c r="N53" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="O53" s="12">
-        <v>0</v>
-      </c>
-      <c r="P53" s="12">
+      <c r="O53" s="11">
+        <v>0</v>
+      </c>
+      <c r="P53" s="11">
         <v>1.1389570356218393</v>
       </c>
-      <c r="Q53" s="12">
+      <c r="Q53" s="11">
         <v>1.0544300539232154</v>
       </c>
-      <c r="R53" s="12">
+      <c r="R53" s="11">
         <v>1.0047202646085629</v>
       </c>
-      <c r="S53" s="12">
+      <c r="S53" s="11">
         <v>0.93836331315770904</v>
       </c>
-      <c r="T53" s="12">
+      <c r="T53" s="11">
         <v>0.89878949162663713</v>
       </c>
     </row>
@@ -3087,22 +3275,22 @@
       <c r="N54" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="O54" s="12">
-        <v>0</v>
-      </c>
-      <c r="P54" s="12">
+      <c r="O54" s="11">
+        <v>0</v>
+      </c>
+      <c r="P54" s="11">
         <v>-1553.6739736999996</v>
       </c>
-      <c r="Q54" s="12">
+      <c r="Q54" s="11">
         <v>4336.4969207500999</v>
       </c>
-      <c r="R54" s="12">
+      <c r="R54" s="11">
         <v>4336.6108503835003</v>
       </c>
-      <c r="S54" s="12">
+      <c r="S54" s="11">
         <v>4336.7817448336</v>
       </c>
-      <c r="T54" s="12">
+      <c r="T54" s="11">
         <v>4336.8956744670004</v>
       </c>
     </row>
@@ -3110,22 +3298,22 @@
       <c r="N55" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="O55" s="12">
-        <v>0</v>
-      </c>
-      <c r="P55" s="12">
+      <c r="O55" s="11">
+        <v>0</v>
+      </c>
+      <c r="P55" s="11">
         <v>-28.113149870868526</v>
       </c>
-      <c r="Q55" s="12">
+      <c r="Q55" s="11">
         <v>72.643890257327683</v>
       </c>
-      <c r="R55" s="12">
+      <c r="R55" s="11">
         <v>69.22100323188468</v>
       </c>
-      <c r="S55" s="12">
+      <c r="S55" s="11">
         <v>64.651835844524058</v>
       </c>
-      <c r="T55" s="12">
+      <c r="T55" s="11">
         <v>61.926885243577217</v>
       </c>
     </row>
@@ -3133,22 +3321,22 @@
       <c r="N56" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="O56" s="12">
+      <c r="O56" s="11">
         <v>860.14626825458322</v>
       </c>
-      <c r="P56" s="12">
+      <c r="P56" s="11">
         <v>206.8726634074329</v>
       </c>
-      <c r="Q56" s="12">
+      <c r="Q56" s="11">
         <v>147.80162343445511</v>
       </c>
-      <c r="R56" s="12">
+      <c r="R56" s="11">
         <v>108.42093011913654</v>
       </c>
-      <c r="S56" s="12">
+      <c r="S56" s="11">
         <v>49.349890146158721</v>
       </c>
-      <c r="T56" s="12">
+      <c r="T56" s="11">
         <v>9.9691968308401844</v>
       </c>
     </row>
@@ -3156,27 +3344,35 @@
       <c r="N57" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="O57" s="12">
+      <c r="O57" s="11">
         <v>3207.9471826351819</v>
       </c>
-      <c r="P57" s="12">
+      <c r="P57" s="11">
         <v>4047.5944455509716</v>
       </c>
-      <c r="Q57" s="12">
+      <c r="Q57" s="11">
         <v>4047.5944455509716</v>
       </c>
-      <c r="R57" s="12">
+      <c r="R57" s="11">
         <v>4047.5944455509716</v>
       </c>
-      <c r="S57" s="12">
+      <c r="S57" s="11">
         <v>4047.5944455509716</v>
       </c>
-      <c r="T57" s="12">
+      <c r="T57" s="11">
         <v>4047.5944455509716</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A14:G14"/>
+    <mergeCell ref="A15:B18"/>
+    <mergeCell ref="C15:G15"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="D17:D18"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="G17:G18"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:B5"/>
     <mergeCell ref="C2:G2"/>
@@ -3185,14 +3381,6 @@
     <mergeCell ref="E4:E5"/>
     <mergeCell ref="F4:F5"/>
     <mergeCell ref="G4:G5"/>
-    <mergeCell ref="A14:G14"/>
-    <mergeCell ref="A15:B18"/>
-    <mergeCell ref="C15:G15"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="D17:D18"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="G17:G18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
made range bigger to accomodate robilante
</commit_message>
<xml_diff>
--- a/adopt_net0/database/templates/technology_data/Industrial/CementHybridCCS_data/cement_sheet.xlsx
+++ b/adopt_net0/database/templates/technology_data/Industrial/CementHybridCCS_data/cement_sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\0954659\PycharmProjects\AdOpT-NET0_luca\adopt_net0\database\templates\technology_data\Industrial\CementHybridCCS_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D196E75-67D7-46C5-8F2F-B7E942B46090}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0064542-306E-4AE4-8E2A-76DCB265744D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C0ECAA26-0769-408D-9398-31AECF4E3649}"/>
   </bookViews>
@@ -777,6 +777,7 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="13" xfId="4" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="13" xfId="4" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -813,7 +814,6 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="3" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Calculation" xfId="5" builtinId="22"/>
@@ -1207,12 +1207,12 @@
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" s="33">
-        <v>200</v>
-      </c>
-      <c r="B4" s="33">
+      <c r="A4" s="21">
+        <v>220</v>
+      </c>
+      <c r="B4" s="21">
         <f>_xlfn.FORECAST.LINEAR($A$4, B2:B3, $A$2:$A$3)</f>
-        <v>104735000</v>
+        <v>113371000</v>
       </c>
     </row>
   </sheetData>
@@ -1273,10 +1273,10 @@
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="33">
+      <c r="A5" s="21">
         <v>50</v>
       </c>
-      <c r="B5" s="33">
+      <c r="B5" s="21">
         <f>_xlfn.FORECAST.LINEAR($A$5, B3:B4, $A$3:$A$4)</f>
         <v>30689778.48449932</v>
       </c>
@@ -1350,20 +1350,20 @@
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="33">
-        <v>200</v>
-      </c>
-      <c r="B5" s="33">
+      <c r="A5" s="21">
+        <v>220</v>
+      </c>
+      <c r="B5" s="21">
         <f>_xlfn.FORECAST.LINEAR($A$5, B3:B4, $A$3:$A$4)</f>
-        <v>83350000</v>
-      </c>
-      <c r="C5" s="33">
+        <v>88910000</v>
+      </c>
+      <c r="C5" s="21">
         <f t="shared" ref="C5:D5" si="0">_xlfn.FORECAST.LINEAR($A$5, C3:C4, $A$3:$A$4)</f>
-        <v>82950000</v>
-      </c>
-      <c r="D5" s="33">
+        <v>88190000</v>
+      </c>
+      <c r="D5" s="21">
         <f t="shared" si="0"/>
-        <v>87500000</v>
+        <v>91740000</v>
       </c>
     </row>
   </sheetData>
@@ -1465,18 +1465,18 @@
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="33">
+      <c r="A6" s="21">
         <v>50</v>
       </c>
-      <c r="B6" s="33">
+      <c r="B6" s="21">
         <f>_xlfn.FORECAST.LINEAR($A$6, B4:B5, A4:A5)</f>
         <v>18648960.688236542</v>
       </c>
-      <c r="C6" s="33">
+      <c r="C6" s="21">
         <f>_xlfn.FORECAST.LINEAR($A$6, C4:C5, A4:A5)</f>
         <v>21918026.046032257</v>
       </c>
-      <c r="D6" s="33">
+      <c r="D6" s="21">
         <f>_xlfn.FORECAST.LINEAR($A$6, D4:D5, A4:A5)</f>
         <v>28821920.599393677</v>
       </c>
@@ -1615,15 +1615,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="16.2" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="23"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="24"/>
       <c r="N1" s="10"/>
       <c r="O1" s="10" t="s">
         <v>40</v>
@@ -1635,17 +1635,17 @@
       <c r="T1" s="3"/>
     </row>
     <row r="2" spans="1:20" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="30" t="s">
+      <c r="B2" s="26"/>
+      <c r="C2" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="32"/>
       <c r="N2" s="3"/>
       <c r="O2" s="3" t="s">
         <v>17</v>
@@ -1667,8 +1667,8 @@
       </c>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A3" s="26"/>
-      <c r="B3" s="27"/>
+      <c r="A3" s="27"/>
+      <c r="B3" s="28"/>
       <c r="C3" s="1" t="s">
         <v>6</v>
       </c>
@@ -1707,21 +1707,21 @@
       </c>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A4" s="26"/>
-      <c r="B4" s="27"/>
-      <c r="C4" s="32">
+      <c r="A4" s="27"/>
+      <c r="B4" s="28"/>
+      <c r="C4" s="33">
         <v>72.349999999999994</v>
       </c>
-      <c r="D4" s="32">
+      <c r="D4" s="33">
         <v>84.320988516056687</v>
       </c>
-      <c r="E4" s="32">
+      <c r="E4" s="33">
         <v>89.206549352337717</v>
       </c>
-      <c r="F4" s="32">
+      <c r="F4" s="33">
         <v>95.445590190807295</v>
       </c>
-      <c r="G4" s="32">
+      <c r="G4" s="33">
         <v>99.17</v>
       </c>
       <c r="N4" s="3" t="s">
@@ -1747,13 +1747,13 @@
       </c>
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A5" s="28"/>
-      <c r="B5" s="29"/>
-      <c r="C5" s="32"/>
-      <c r="D5" s="32"/>
-      <c r="E5" s="32"/>
-      <c r="F5" s="32"/>
-      <c r="G5" s="32"/>
+      <c r="A5" s="29"/>
+      <c r="B5" s="30"/>
+      <c r="C5" s="33"/>
+      <c r="D5" s="33"/>
+      <c r="E5" s="33"/>
+      <c r="F5" s="33"/>
+      <c r="G5" s="33"/>
       <c r="L5">
         <f>1-P6/P5</f>
         <v>0.78184911505744248</v>
@@ -2114,15 +2114,15 @@
       </c>
     </row>
     <row r="14" spans="1:20" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A14" s="21" t="s">
+      <c r="A14" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="22"/>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="22"/>
-      <c r="G14" s="23"/>
+      <c r="B14" s="23"/>
+      <c r="C14" s="23"/>
+      <c r="D14" s="23"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="23"/>
+      <c r="G14" s="24"/>
       <c r="N14" s="3" t="s">
         <v>29</v>
       </c>
@@ -2146,17 +2146,17 @@
       </c>
     </row>
     <row r="15" spans="1:20" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A15" s="24" t="s">
+      <c r="A15" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="B15" s="25"/>
-      <c r="C15" s="30" t="s">
+      <c r="B15" s="26"/>
+      <c r="C15" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="D15" s="30"/>
-      <c r="E15" s="30"/>
-      <c r="F15" s="30"/>
-      <c r="G15" s="31"/>
+      <c r="D15" s="31"/>
+      <c r="E15" s="31"/>
+      <c r="F15" s="31"/>
+      <c r="G15" s="32"/>
       <c r="N15" s="3" t="s">
         <v>30</v>
       </c>
@@ -2180,8 +2180,8 @@
       </c>
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A16" s="26"/>
-      <c r="B16" s="27"/>
+      <c r="A16" s="27"/>
+      <c r="B16" s="28"/>
       <c r="C16" s="1" t="s">
         <v>6</v>
       </c>
@@ -2220,21 +2220,21 @@
       </c>
     </row>
     <row r="17" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A17" s="26"/>
-      <c r="B17" s="27"/>
-      <c r="C17" s="32">
+      <c r="A17" s="27"/>
+      <c r="B17" s="28"/>
+      <c r="C17" s="33">
         <v>50.76</v>
       </c>
-      <c r="D17" s="32">
+      <c r="D17" s="33">
         <v>64.722331812465825</v>
       </c>
-      <c r="E17" s="32">
+      <c r="E17" s="33">
         <v>68.47234583745032</v>
       </c>
-      <c r="F17" s="32">
+      <c r="F17" s="33">
         <v>73.261251641870047</v>
       </c>
-      <c r="G17" s="32">
+      <c r="G17" s="33">
         <v>76.12</v>
       </c>
       <c r="N17" s="3" t="s">
@@ -2260,13 +2260,13 @@
       </c>
     </row>
     <row r="18" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A18" s="28"/>
-      <c r="B18" s="29"/>
-      <c r="C18" s="32"/>
-      <c r="D18" s="32"/>
-      <c r="E18" s="32"/>
-      <c r="F18" s="32"/>
-      <c r="G18" s="32"/>
+      <c r="A18" s="29"/>
+      <c r="B18" s="30"/>
+      <c r="C18" s="33"/>
+      <c r="D18" s="33"/>
+      <c r="E18" s="33"/>
+      <c r="F18" s="33"/>
+      <c r="G18" s="33"/>
       <c r="N18" s="3" t="s">
         <v>33</v>
       </c>
@@ -3365,6 +3365,14 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:B5"/>
+    <mergeCell ref="C2:G2"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="F4:F5"/>
+    <mergeCell ref="G4:G5"/>
     <mergeCell ref="A14:G14"/>
     <mergeCell ref="A15:B18"/>
     <mergeCell ref="C15:G15"/>
@@ -3373,14 +3381,6 @@
     <mergeCell ref="E17:E18"/>
     <mergeCell ref="F17:F18"/>
     <mergeCell ref="G17:G18"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:B5"/>
-    <mergeCell ref="C2:G2"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="F4:F5"/>
-    <mergeCell ref="G4:G5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>